<commit_message>
Changement des plans sur altium.
J'ai du changer les plans en 2 plans de masse. J'ai donc du refaire une partie du routage pour corriger cette erreur. -> j'avais a plan de masse et 1 plan de VCC avant.
</commit_message>
<xml_diff>
--- a/jeu_du_moulin_boura/rpt/jeu-du-moulin-bourquenouda-rpt-journal.xlsx
+++ b/jeu_du_moulin_boura/rpt/jeu-du-moulin-bourquenouda-rpt-journal.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/alexandre_bourquenoud_studentfr_ch/Documents/PHIE/jeu_du_moulin_alexandre_bourquenoud/jeu_du_moulin_2025_boura/jeu_du_moulin_boura/rpt/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bourquenouda01\OneDrive - EDUETATFR\PHIE\jeu_du_moulin_alexandre_bourquenoud\jeu_du_moulin_2025_boura\jeu_du_moulin_boura\rpt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="13_ncr:1_{5F77AD1B-655E-40F7-81BC-FD86898DA849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85A58703-8C08-45C7-A6BE-FC048B19116A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED970C68-2653-443C-99A4-F9D694477206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="s1" sheetId="8" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="68">
   <si>
     <t>Date</t>
   </si>
@@ -287,6 +287,32 @@
   </si>
   <si>
     <t xml:space="preserve"> Pour cette première semaine, je pense avoir bien travailler avec  un nombre minime de problèmes rencontré même si je devrais prendre plus de temps a rédiger la documentation mais je peux quand même dire que j'ai un peu d'avance dans le routage malgré une petite confusion qui n'est pas encore résolue. Les changements engendré par cette confusion ne seront pas trop élevé je pense donc même si le routage doit être changé, ça ne prendra pas trop de temps.</t>
+  </si>
+  <si>
+    <t>rédaction du journal de travail.</t>
+  </si>
+  <si>
+    <t>fin de création de la BOM complète et commande des composants qui ne sont pas disponible à l'atelier</t>
+  </si>
+  <si>
+    <t>Changement  "fondamental" du circuit. En effet, a cause d'un problème de compréhension, j'avais utiliser un plan de masse et un plan de VCC alors qu'il fallait plan de masse. Je dois donc changer le routage pour remédier a ce problème</t>
+  </si>
+  <si>
+    <t>rédaction de la documentation -&gt; ajout des commentaire au sujet du placement des composants</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Je n'ai pas pu ajouté le silkscreen au sommet des touches -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>Je demanderai a M. Egli car il a des meilleur connaissances sur altium.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -564,6 +590,18 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -599,18 +637,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -987,10 +1013,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
@@ -1294,19 +1316,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="36" t="s">
+      <c r="D3" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="38" t="s">
+      <c r="E3" s="42" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -1317,11 +1339,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="36"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="38"/>
+      <c r="A4" s="40"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="42"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -1330,7 +1352,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" s="10" customFormat="1" ht="78.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="39" t="s">
+      <c r="A5" s="43" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -1350,8 +1372,8 @@
       </c>
       <c r="G5" s="14"/>
     </row>
-    <row r="6" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A6" s="40"/>
+    <row r="6" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
+      <c r="A6" s="44"/>
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
@@ -1368,7 +1390,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="40"/>
+      <c r="A7" s="44"/>
       <c r="B7" s="5" t="s">
         <v>22</v>
       </c>
@@ -1387,7 +1409,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="40"/>
+      <c r="A8" s="44"/>
       <c r="B8" s="5" t="s">
         <v>22</v>
       </c>
@@ -1404,7 +1426,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A9" s="40"/>
+      <c r="A9" s="44"/>
       <c r="B9" s="5" t="s">
         <v>22</v>
       </c>
@@ -1421,7 +1443,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" s="10" customFormat="1" ht="78.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="40"/>
+      <c r="A10" s="44"/>
       <c r="B10" s="5" t="s">
         <v>22</v>
       </c>
@@ -1440,7 +1462,7 @@
       <c r="G10" s="14"/>
     </row>
     <row r="11" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A11" s="40"/>
+      <c r="A11" s="44"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -1465,7 +1487,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A13" s="43" t="s">
+      <c r="A13" s="47" t="s">
         <v>5</v>
       </c>
       <c r="B13" s="5" t="s">
@@ -1484,7 +1506,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A14" s="44"/>
+      <c r="A14" s="48"/>
       <c r="B14" s="5" t="s">
         <v>22</v>
       </c>
@@ -1501,7 +1523,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="44"/>
+      <c r="A15" s="48"/>
       <c r="B15" s="5" t="s">
         <v>22</v>
       </c>
@@ -1518,7 +1540,7 @@
       <c r="G15" s="14"/>
     </row>
     <row r="16" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A16" s="44"/>
+      <c r="A16" s="48"/>
       <c r="B16" s="5" t="s">
         <v>22</v>
       </c>
@@ -1535,7 +1557,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A17" s="44"/>
+      <c r="A17" s="48"/>
       <c r="B17" s="5" t="s">
         <v>22</v>
       </c>
@@ -1552,7 +1574,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="44"/>
+      <c r="A18" s="48"/>
       <c r="B18" s="5" t="s">
         <v>22</v>
       </c>
@@ -1569,7 +1591,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A19" s="44"/>
+      <c r="A19" s="48"/>
       <c r="B19" s="5"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -1594,7 +1616,7 @@
       <c r="G20" s="14"/>
     </row>
     <row r="21" spans="1:7" s="10" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
-      <c r="A21" s="39" t="s">
+      <c r="A21" s="43" t="s">
         <v>7</v>
       </c>
       <c r="B21" s="5" t="s">
@@ -1613,7 +1635,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="40"/>
+      <c r="A22" s="44"/>
       <c r="B22" s="5" t="s">
         <v>22</v>
       </c>
@@ -1629,8 +1651,8 @@
       </c>
       <c r="G22" s="14"/>
     </row>
-    <row r="23" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A23" s="40"/>
+    <row r="23" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
+      <c r="A23" s="44"/>
       <c r="B23" s="5" t="s">
         <v>22</v>
       </c>
@@ -1647,7 +1669,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A24" s="40"/>
+      <c r="A24" s="44"/>
       <c r="B24" s="5" t="s">
         <v>22</v>
       </c>
@@ -1664,7 +1686,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A25" s="40"/>
+      <c r="A25" s="44"/>
       <c r="B25" s="5" t="s">
         <v>22</v>
       </c>
@@ -1681,7 +1703,7 @@
       <c r="G25" s="14"/>
     </row>
     <row r="26" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="40"/>
+      <c r="A26" s="44"/>
       <c r="B26" s="5" t="s">
         <v>22</v>
       </c>
@@ -1700,7 +1722,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A27" s="40"/>
+      <c r="A27" s="44"/>
       <c r="B27" s="5" t="s">
         <v>22</v>
       </c>
@@ -1732,8 +1754,8 @@
       </c>
       <c r="G28" s="14"/>
     </row>
-    <row r="29" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A29" s="39" t="s">
+    <row r="29" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
+      <c r="A29" s="43" t="s">
         <v>8</v>
       </c>
       <c r="B29" s="5" t="s">
@@ -1752,7 +1774,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A30" s="40"/>
+      <c r="A30" s="44"/>
       <c r="B30" s="5" t="s">
         <v>22</v>
       </c>
@@ -1771,7 +1793,7 @@
       <c r="G30" s="14"/>
     </row>
     <row r="31" spans="1:7" s="10" customFormat="1" ht="90" x14ac:dyDescent="0.2">
-      <c r="A31" s="40"/>
+      <c r="A31" s="44"/>
       <c r="B31" s="5" t="s">
         <v>22</v>
       </c>
@@ -1790,7 +1812,7 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" s="10" customFormat="1" ht="78.75" x14ac:dyDescent="0.2">
-      <c r="A32" s="40"/>
+      <c r="A32" s="44"/>
       <c r="B32" s="5" t="s">
         <v>22</v>
       </c>
@@ -1807,7 +1829,7 @@
       <c r="G32" s="14"/>
     </row>
     <row r="33" spans="1:7" s="10" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
-      <c r="A33" s="40"/>
+      <c r="A33" s="44"/>
       <c r="B33" s="5" t="s">
         <v>22</v>
       </c>
@@ -1824,7 +1846,7 @@
       <c r="G33" s="14"/>
     </row>
     <row r="34" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A34" s="40"/>
+      <c r="A34" s="44"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
@@ -1850,8 +1872,8 @@
       </c>
       <c r="G35" s="14"/>
     </row>
-    <row r="36" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A36" s="39" t="s">
+    <row r="36" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
+      <c r="A36" s="43" t="s">
         <v>9</v>
       </c>
       <c r="B36" s="5" t="s">
@@ -1870,7 +1892,7 @@
       <c r="G36" s="14"/>
     </row>
     <row r="37" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A37" s="40"/>
+      <c r="A37" s="44"/>
       <c r="B37" s="5" t="s">
         <v>22</v>
       </c>
@@ -1885,7 +1907,7 @@
       <c r="G37" s="14"/>
     </row>
     <row r="38" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A38" s="40"/>
+      <c r="A38" s="44"/>
       <c r="B38" s="5" t="s">
         <v>22</v>
       </c>
@@ -1904,7 +1926,7 @@
       <c r="G38" s="14"/>
     </row>
     <row r="39" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A39" s="40"/>
+      <c r="A39" s="44"/>
       <c r="B39" s="5" t="s">
         <v>22</v>
       </c>
@@ -1923,7 +1945,7 @@
       <c r="G39" s="14"/>
     </row>
     <row r="40" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A40" s="40"/>
+      <c r="A40" s="44"/>
       <c r="B40" s="5"/>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
@@ -1948,12 +1970,12 @@
       <c r="G41" s="14"/>
     </row>
     <row r="42" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="38" t="s">
+      <c r="A42" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="B42" s="41"/>
-      <c r="C42" s="41"/>
-      <c r="D42" s="42"/>
+      <c r="B42" s="45"/>
+      <c r="C42" s="45"/>
+      <c r="D42" s="46"/>
       <c r="E42" s="17"/>
       <c r="F42" s="17" t="s">
         <v>12</v>
@@ -1964,36 +1986,36 @@
       </c>
     </row>
     <row r="43" spans="1:7" s="10" customFormat="1" ht="82.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="33" t="s">
+      <c r="A43" s="37" t="s">
         <v>62</v>
       </c>
-      <c r="B43" s="34"/>
-      <c r="C43" s="34"/>
-      <c r="D43" s="34"/>
-      <c r="E43" s="34"/>
-      <c r="F43" s="34"/>
-      <c r="G43" s="35"/>
+      <c r="B43" s="38"/>
+      <c r="C43" s="38"/>
+      <c r="D43" s="38"/>
+      <c r="E43" s="38"/>
+      <c r="F43" s="38"/>
+      <c r="G43" s="39"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="45"/>
-      <c r="B46" s="45"/>
-      <c r="C46" s="46"/>
-      <c r="D46" s="45"/>
-      <c r="E46" s="45"/>
+      <c r="A46" s="34"/>
+      <c r="B46" s="34"/>
+      <c r="C46" s="36"/>
+      <c r="D46" s="34"/>
+      <c r="E46" s="34"/>
       <c r="F46" s="23"/>
       <c r="G46" s="23"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="45"/>
-      <c r="B47" s="45"/>
-      <c r="C47" s="46"/>
-      <c r="D47" s="45"/>
-      <c r="E47" s="45"/>
+      <c r="A47" s="34"/>
+      <c r="B47" s="34"/>
+      <c r="C47" s="36"/>
+      <c r="D47" s="34"/>
+      <c r="E47" s="34"/>
       <c r="F47" s="23"/>
       <c r="G47" s="23"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="47"/>
+      <c r="A48" s="33"/>
       <c r="B48" s="25"/>
       <c r="C48" s="25"/>
       <c r="D48" s="25"/>
@@ -2002,7 +2024,7 @@
       <c r="G48" s="10"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="47"/>
+      <c r="A49" s="33"/>
       <c r="B49" s="25"/>
       <c r="C49" s="25"/>
       <c r="D49" s="25"/>
@@ -2011,7 +2033,7 @@
       <c r="G49" s="10"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="47"/>
+      <c r="A50" s="33"/>
       <c r="B50" s="25"/>
       <c r="C50" s="25"/>
       <c r="D50" s="25"/>
@@ -2020,7 +2042,7 @@
       <c r="G50" s="10"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="47"/>
+      <c r="A51" s="33"/>
       <c r="B51" s="25"/>
       <c r="C51" s="25"/>
       <c r="D51" s="25"/>
@@ -2029,7 +2051,7 @@
       <c r="G51" s="10"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="47"/>
+      <c r="A52" s="33"/>
       <c r="B52" s="25"/>
       <c r="C52" s="25"/>
       <c r="D52" s="25"/>
@@ -2038,7 +2060,7 @@
       <c r="G52" s="10"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="47"/>
+      <c r="A53" s="33"/>
       <c r="B53" s="25"/>
       <c r="C53" s="25"/>
       <c r="D53" s="25"/>
@@ -2056,7 +2078,7 @@
       <c r="G54" s="10"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="47"/>
+      <c r="A55" s="33"/>
       <c r="B55" s="25"/>
       <c r="C55" s="25"/>
       <c r="D55" s="25"/>
@@ -2065,7 +2087,7 @@
       <c r="G55" s="10"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="47"/>
+      <c r="A56" s="33"/>
       <c r="B56" s="25"/>
       <c r="C56" s="25"/>
       <c r="D56" s="25"/>
@@ -2074,7 +2096,7 @@
       <c r="G56" s="10"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="47"/>
+      <c r="A57" s="33"/>
       <c r="B57" s="25"/>
       <c r="C57" s="25"/>
       <c r="D57" s="25"/>
@@ -2083,7 +2105,7 @@
       <c r="G57" s="10"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="47"/>
+      <c r="A58" s="33"/>
       <c r="B58" s="25"/>
       <c r="C58" s="25"/>
       <c r="D58" s="25"/>
@@ -2101,7 +2123,7 @@
       <c r="G59" s="10"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="47"/>
+      <c r="A60" s="33"/>
       <c r="B60" s="25"/>
       <c r="C60" s="25"/>
       <c r="D60" s="25"/>
@@ -2110,7 +2132,7 @@
       <c r="G60" s="10"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="47"/>
+      <c r="A61" s="33"/>
       <c r="B61" s="25"/>
       <c r="C61" s="25"/>
       <c r="D61" s="25"/>
@@ -2119,7 +2141,7 @@
       <c r="G61" s="10"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="47"/>
+      <c r="A62" s="33"/>
       <c r="B62" s="25"/>
       <c r="C62" s="25"/>
       <c r="D62" s="25"/>
@@ -2128,7 +2150,7 @@
       <c r="G62" s="10"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="47"/>
+      <c r="A63" s="33"/>
       <c r="B63" s="25"/>
       <c r="C63" s="25"/>
       <c r="D63" s="25"/>
@@ -2146,7 +2168,7 @@
       <c r="G64" s="10"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" s="47"/>
+      <c r="A65" s="33"/>
       <c r="B65" s="25"/>
       <c r="C65" s="25"/>
       <c r="D65" s="25"/>
@@ -2155,7 +2177,7 @@
       <c r="G65" s="10"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" s="47"/>
+      <c r="A66" s="33"/>
       <c r="B66" s="25"/>
       <c r="C66" s="25"/>
       <c r="D66" s="25"/>
@@ -2164,7 +2186,7 @@
       <c r="G66" s="10"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" s="47"/>
+      <c r="A67" s="33"/>
       <c r="B67" s="25"/>
       <c r="C67" s="25"/>
       <c r="D67" s="25"/>
@@ -2173,7 +2195,7 @@
       <c r="G67" s="10"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" s="47"/>
+      <c r="A68" s="33"/>
       <c r="B68" s="25"/>
       <c r="C68" s="25"/>
       <c r="D68" s="25"/>
@@ -2191,7 +2213,7 @@
       <c r="G69" s="10"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" s="47"/>
+      <c r="A70" s="33"/>
       <c r="B70" s="25"/>
       <c r="C70" s="25"/>
       <c r="D70" s="25"/>
@@ -2200,7 +2222,7 @@
       <c r="G70" s="10"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" s="47"/>
+      <c r="A71" s="33"/>
       <c r="B71" s="25"/>
       <c r="C71" s="25"/>
       <c r="D71" s="25"/>
@@ -2209,7 +2231,7 @@
       <c r="G71" s="10"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" s="47"/>
+      <c r="A72" s="33"/>
       <c r="B72" s="25"/>
       <c r="C72" s="25"/>
       <c r="D72" s="25"/>
@@ -2218,7 +2240,7 @@
       <c r="G72" s="10"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A73" s="47"/>
+      <c r="A73" s="33"/>
       <c r="B73" s="25"/>
       <c r="C73" s="25"/>
       <c r="D73" s="25"/>
@@ -2236,37 +2258,25 @@
       <c r="G74" s="10"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" s="45"/>
-      <c r="B75" s="45"/>
-      <c r="C75" s="45"/>
-      <c r="D75" s="45"/>
+      <c r="A75" s="34"/>
+      <c r="B75" s="34"/>
+      <c r="C75" s="34"/>
+      <c r="D75" s="34"/>
       <c r="E75" s="27"/>
       <c r="F75" s="27"/>
       <c r="G75" s="28"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" s="48"/>
-      <c r="B76" s="48"/>
-      <c r="C76" s="48"/>
-      <c r="D76" s="48"/>
-      <c r="E76" s="48"/>
-      <c r="F76" s="48"/>
-      <c r="G76" s="48"/>
+      <c r="A76" s="35"/>
+      <c r="B76" s="35"/>
+      <c r="C76" s="35"/>
+      <c r="D76" s="35"/>
+      <c r="E76" s="35"/>
+      <c r="F76" s="35"/>
+      <c r="G76" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A48:A53"/>
-    <mergeCell ref="A75:D75"/>
-    <mergeCell ref="A76:G76"/>
-    <mergeCell ref="A55:A58"/>
-    <mergeCell ref="A60:A63"/>
-    <mergeCell ref="A65:A68"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A46:A47"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="E46:E47"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
@@ -2279,6 +2289,18 @@
     <mergeCell ref="A36:A40"/>
     <mergeCell ref="A42:D42"/>
     <mergeCell ref="A13:A19"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="E46:E47"/>
+    <mergeCell ref="A48:A53"/>
+    <mergeCell ref="A75:D75"/>
+    <mergeCell ref="A76:G76"/>
+    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="A60:A63"/>
+    <mergeCell ref="A65:A68"/>
+    <mergeCell ref="A70:A73"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F16 F20:F41">
     <cfRule type="containsText" dxfId="31" priority="1" operator="containsText" text="Terminé">
@@ -2359,19 +2381,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="36" t="s">
+      <c r="D3" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="38" t="s">
+      <c r="E3" s="42" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -2382,11 +2404,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="36"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="38"/>
+      <c r="A4" s="40"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="42"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -2394,46 +2416,80 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A5" s="39" t="s">
+    <row r="5" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
+      <c r="A5" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
+      <c r="B5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="E5" s="4"/>
-      <c r="F5" s="13"/>
+      <c r="F5" s="13">
+        <v>0.2</v>
+      </c>
       <c r="G5" s="14"/>
     </row>
-    <row r="6" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A6" s="40"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
+    <row r="6" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+      <c r="A6" s="44"/>
+      <c r="B6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>64</v>
+      </c>
       <c r="E6" s="5"/>
-      <c r="F6" s="13"/>
+      <c r="F6" s="13">
+        <v>2</v>
+      </c>
       <c r="G6" s="14"/>
     </row>
-    <row r="7" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A7" s="40"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="13"/>
+    <row r="7" spans="1:7" s="10" customFormat="1" ht="90" x14ac:dyDescent="0.2">
+      <c r="A7" s="44"/>
+      <c r="B7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F7" s="13">
+        <v>3.8</v>
+      </c>
       <c r="G7" s="14"/>
     </row>
-    <row r="8" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="40"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+    <row r="8" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="44"/>
+      <c r="B8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>66</v>
+      </c>
       <c r="E8" s="4"/>
-      <c r="F8" s="6"/>
+      <c r="F8" s="6">
+        <v>1</v>
+      </c>
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="40"/>
+      <c r="A9" s="44"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -2442,7 +2498,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="40"/>
+      <c r="A10" s="44"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -2451,8 +2507,8 @@
       <c r="G10" s="14"/>
     </row>
     <row r="11" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A11" s="15" t="s">
-        <v>21</v>
+      <c r="A11" s="31">
+        <v>45796</v>
       </c>
       <c r="B11" s="16"/>
       <c r="C11" s="16"/>
@@ -2462,12 +2518,12 @@
       </c>
       <c r="F11" s="18">
         <f>SUM(F5:F10)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A12" s="40" t="s">
+      <c r="A12" s="44" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -2478,7 +2534,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A13" s="40"/>
+      <c r="A13" s="44"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -2487,7 +2543,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A14" s="40"/>
+      <c r="A14" s="44"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -2496,7 +2552,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="40"/>
+      <c r="A15" s="44"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -2506,7 +2562,7 @@
     </row>
     <row r="16" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
       <c r="A16" s="31">
-        <v>45301</v>
+        <v>45797</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="16"/>
@@ -2521,7 +2577,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A17" s="40" t="s">
+      <c r="A17" s="44" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -2533,7 +2589,7 @@
       <c r="J17" s="32"/>
     </row>
     <row r="18" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A18" s="40"/>
+      <c r="A18" s="44"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -2542,7 +2598,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A19" s="40"/>
+      <c r="A19" s="44"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -2551,7 +2607,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="40"/>
+      <c r="A20" s="44"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -2561,7 +2617,7 @@
     </row>
     <row r="21" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
       <c r="A21" s="31">
-        <v>45332</v>
+        <v>45798</v>
       </c>
       <c r="B21" s="16"/>
       <c r="C21" s="16"/>
@@ -2576,7 +2632,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A22" s="40" t="s">
+      <c r="A22" s="44" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -2587,7 +2643,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A23" s="40"/>
+      <c r="A23" s="44"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -2597,7 +2653,7 @@
       <c r="J23" s="32"/>
     </row>
     <row r="24" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A24" s="40"/>
+      <c r="A24" s="44"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -2607,7 +2663,7 @@
       <c r="J24" s="32"/>
     </row>
     <row r="25" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="40"/>
+      <c r="A25" s="44"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -2617,7 +2673,7 @@
     </row>
     <row r="26" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
       <c r="A26" s="31">
-        <v>45361</v>
+        <v>45799</v>
       </c>
       <c r="B26" s="16"/>
       <c r="C26" s="16"/>
@@ -2632,7 +2688,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A27" s="40" t="s">
+      <c r="A27" s="44" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -2643,7 +2699,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A28" s="40"/>
+      <c r="A28" s="44"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -2652,7 +2708,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A29" s="40"/>
+      <c r="A29" s="44"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -2661,7 +2717,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="40"/>
+      <c r="A30" s="44"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -2671,7 +2727,7 @@
     </row>
     <row r="31" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="31">
-        <v>45392</v>
+        <v>45800</v>
       </c>
       <c r="B31" s="19"/>
       <c r="C31" s="19"/>
@@ -2686,31 +2742,31 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:10" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="36" t="s">
+      <c r="A32" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="36"/>
-      <c r="C32" s="36"/>
-      <c r="D32" s="36"/>
+      <c r="B32" s="40"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="40"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
       </c>
       <c r="G32" s="22">
         <f>F11+F16+F21+F26+F31</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="33" t="s">
+      <c r="A33" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="34"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="34"/>
-      <c r="G33" s="35"/>
+      <c r="B33" s="38"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -2785,19 +2841,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="36" t="s">
+      <c r="D3" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="38" t="s">
+      <c r="E3" s="42" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -2808,11 +2864,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="36"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="38"/>
+      <c r="A4" s="40"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="42"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -2821,7 +2877,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="39" t="s">
+      <c r="A5" s="43" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -2832,7 +2888,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="40"/>
+      <c r="A6" s="44"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -2841,7 +2897,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="40"/>
+      <c r="A7" s="44"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -2850,7 +2906,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="40"/>
+      <c r="A8" s="44"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -2859,7 +2915,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="40"/>
+      <c r="A9" s="44"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -2868,7 +2924,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="40"/>
+      <c r="A10" s="44"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -2893,7 +2949,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="40" t="s">
+      <c r="A12" s="44" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -2904,7 +2960,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="40"/>
+      <c r="A13" s="44"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -2913,7 +2969,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="40"/>
+      <c r="A14" s="44"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -2922,7 +2978,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="40"/>
+      <c r="A15" s="44"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -2947,7 +3003,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="40" t="s">
+      <c r="A17" s="44" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -2958,7 +3014,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="40"/>
+      <c r="A18" s="44"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -2967,7 +3023,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="40"/>
+      <c r="A19" s="44"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -2976,7 +3032,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="40"/>
+      <c r="A20" s="44"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -3001,7 +3057,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="40" t="s">
+      <c r="A22" s="44" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -3012,7 +3068,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="40"/>
+      <c r="A23" s="44"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -3021,7 +3077,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="40"/>
+      <c r="A24" s="44"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -3030,7 +3086,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="40"/>
+      <c r="A25" s="44"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -3055,7 +3111,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="40" t="s">
+      <c r="A27" s="44" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -3066,7 +3122,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="40"/>
+      <c r="A28" s="44"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -3075,7 +3131,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="40"/>
+      <c r="A29" s="44"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -3084,7 +3140,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="40"/>
+      <c r="A30" s="44"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -3109,12 +3165,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="36" t="s">
+      <c r="A32" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="36"/>
-      <c r="C32" s="36"/>
-      <c r="D32" s="36"/>
+      <c r="B32" s="40"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="40"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -3125,23 +3181,18 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="33" t="s">
+      <c r="A33" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="34"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="34"/>
-      <c r="G33" s="35"/>
+      <c r="B33" s="38"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A5:A10"/>
@@ -3149,6 +3200,11 @@
     <mergeCell ref="A17:A20"/>
     <mergeCell ref="A22:A25"/>
     <mergeCell ref="A27:A30"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F31">
     <cfRule type="containsText" dxfId="19" priority="1" operator="containsText" text="Terminé">
@@ -3206,19 +3262,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="36" t="s">
+      <c r="D3" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="38" t="s">
+      <c r="E3" s="42" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -3229,11 +3285,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="36"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="38"/>
+      <c r="A4" s="40"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="42"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -3242,7 +3298,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="39" t="s">
+      <c r="A5" s="43" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -3253,7 +3309,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="40"/>
+      <c r="A6" s="44"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -3262,7 +3318,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="40"/>
+      <c r="A7" s="44"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -3271,7 +3327,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="40"/>
+      <c r="A8" s="44"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -3280,7 +3336,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="40"/>
+      <c r="A9" s="44"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -3289,7 +3345,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="40"/>
+      <c r="A10" s="44"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -3314,7 +3370,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="40" t="s">
+      <c r="A12" s="44" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -3325,7 +3381,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="40"/>
+      <c r="A13" s="44"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -3334,7 +3390,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="40"/>
+      <c r="A14" s="44"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -3343,7 +3399,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="40"/>
+      <c r="A15" s="44"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -3368,7 +3424,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="40" t="s">
+      <c r="A17" s="44" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -3379,7 +3435,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="40"/>
+      <c r="A18" s="44"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -3388,7 +3444,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="40"/>
+      <c r="A19" s="44"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -3397,7 +3453,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="40"/>
+      <c r="A20" s="44"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -3422,7 +3478,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="40" t="s">
+      <c r="A22" s="44" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -3433,7 +3489,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="40"/>
+      <c r="A23" s="44"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -3442,7 +3498,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="40"/>
+      <c r="A24" s="44"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -3451,7 +3507,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="40"/>
+      <c r="A25" s="44"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -3476,7 +3532,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="40" t="s">
+      <c r="A27" s="44" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -3487,7 +3543,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="40"/>
+      <c r="A28" s="44"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -3496,7 +3552,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="40"/>
+      <c r="A29" s="44"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -3505,7 +3561,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="40"/>
+      <c r="A30" s="44"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -3530,12 +3586,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="36" t="s">
+      <c r="A32" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="36"/>
-      <c r="C32" s="36"/>
-      <c r="D32" s="36"/>
+      <c r="B32" s="40"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="40"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -3546,23 +3602,18 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="33" t="s">
+      <c r="A33" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="34"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="34"/>
-      <c r="G33" s="35"/>
+      <c r="B33" s="38"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A5:A10"/>
@@ -3570,6 +3621,11 @@
     <mergeCell ref="A17:A20"/>
     <mergeCell ref="A22:A25"/>
     <mergeCell ref="A27:A30"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F31">
     <cfRule type="containsText" dxfId="15" priority="1" operator="containsText" text="Terminé">
@@ -3627,19 +3683,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="36" t="s">
+      <c r="D3" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="38" t="s">
+      <c r="E3" s="42" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -3650,11 +3706,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="36"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="38"/>
+      <c r="A4" s="40"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="42"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -3663,7 +3719,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="39" t="s">
+      <c r="A5" s="43" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -3674,7 +3730,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="40"/>
+      <c r="A6" s="44"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -3683,7 +3739,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="40"/>
+      <c r="A7" s="44"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -3692,7 +3748,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="40"/>
+      <c r="A8" s="44"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -3701,7 +3757,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="40"/>
+      <c r="A9" s="44"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -3710,7 +3766,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="40"/>
+      <c r="A10" s="44"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -3735,7 +3791,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="40" t="s">
+      <c r="A12" s="44" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -3746,7 +3802,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="40"/>
+      <c r="A13" s="44"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -3755,7 +3811,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="40"/>
+      <c r="A14" s="44"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -3764,7 +3820,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="40"/>
+      <c r="A15" s="44"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -3789,7 +3845,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="40" t="s">
+      <c r="A17" s="44" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -3800,7 +3856,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="40"/>
+      <c r="A18" s="44"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -3809,7 +3865,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="40"/>
+      <c r="A19" s="44"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -3818,7 +3874,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="40"/>
+      <c r="A20" s="44"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -3843,7 +3899,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="40" t="s">
+      <c r="A22" s="44" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -3854,7 +3910,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="40"/>
+      <c r="A23" s="44"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -3863,7 +3919,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="40"/>
+      <c r="A24" s="44"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -3872,7 +3928,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="40"/>
+      <c r="A25" s="44"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -3897,7 +3953,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="40" t="s">
+      <c r="A27" s="44" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -3908,7 +3964,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="40"/>
+      <c r="A28" s="44"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -3917,7 +3973,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="40"/>
+      <c r="A29" s="44"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -3926,7 +3982,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="40"/>
+      <c r="A30" s="44"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -3951,12 +4007,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="36" t="s">
+      <c r="A32" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="36"/>
-      <c r="C32" s="36"/>
-      <c r="D32" s="36"/>
+      <c r="B32" s="40"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="40"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -3967,15 +4023,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="33" t="s">
+      <c r="A33" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="34"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="34"/>
-      <c r="G33" s="35"/>
+      <c r="B33" s="38"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -4050,19 +4106,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="36" t="s">
+      <c r="D3" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="38" t="s">
+      <c r="E3" s="42" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -4073,11 +4129,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="36"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="38"/>
+      <c r="A4" s="40"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="42"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -4086,7 +4142,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="39" t="s">
+      <c r="A5" s="43" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -4097,7 +4153,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="40"/>
+      <c r="A6" s="44"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -4106,7 +4162,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="40"/>
+      <c r="A7" s="44"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -4115,7 +4171,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="40"/>
+      <c r="A8" s="44"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -4124,7 +4180,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="40"/>
+      <c r="A9" s="44"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -4133,7 +4189,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="40"/>
+      <c r="A10" s="44"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -4158,7 +4214,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="40" t="s">
+      <c r="A12" s="44" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -4169,7 +4225,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="40"/>
+      <c r="A13" s="44"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -4178,7 +4234,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="40"/>
+      <c r="A14" s="44"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -4187,7 +4243,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="40"/>
+      <c r="A15" s="44"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -4212,7 +4268,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="40" t="s">
+      <c r="A17" s="44" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -4223,7 +4279,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="40"/>
+      <c r="A18" s="44"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -4232,7 +4288,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="40"/>
+      <c r="A19" s="44"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -4241,7 +4297,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="40"/>
+      <c r="A20" s="44"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -4266,7 +4322,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="40" t="s">
+      <c r="A22" s="44" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -4277,7 +4333,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="40"/>
+      <c r="A23" s="44"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -4286,7 +4342,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="40"/>
+      <c r="A24" s="44"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -4295,7 +4351,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="40"/>
+      <c r="A25" s="44"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -4320,7 +4376,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="40" t="s">
+      <c r="A27" s="44" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -4331,7 +4387,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="40"/>
+      <c r="A28" s="44"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -4340,7 +4396,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="40"/>
+      <c r="A29" s="44"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -4349,7 +4405,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="40"/>
+      <c r="A30" s="44"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -4374,12 +4430,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="36" t="s">
+      <c r="A32" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="36"/>
-      <c r="C32" s="36"/>
-      <c r="D32" s="36"/>
+      <c r="B32" s="40"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="40"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -4390,15 +4446,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="33" t="s">
+      <c r="A33" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="34"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="34"/>
-      <c r="G33" s="35"/>
+      <c r="B33" s="38"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -4471,19 +4527,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="36" t="s">
+      <c r="D3" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="38" t="s">
+      <c r="E3" s="42" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -4494,11 +4550,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="36"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="38"/>
+      <c r="A4" s="40"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="42"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -4507,7 +4563,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="39" t="s">
+      <c r="A5" s="43" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -4518,7 +4574,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="40"/>
+      <c r="A6" s="44"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -4527,7 +4583,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="40"/>
+      <c r="A7" s="44"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -4536,7 +4592,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="40"/>
+      <c r="A8" s="44"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -4545,7 +4601,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="40"/>
+      <c r="A9" s="44"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -4554,7 +4610,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="40"/>
+      <c r="A10" s="44"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -4579,7 +4635,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="40" t="s">
+      <c r="A12" s="44" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -4590,7 +4646,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="40"/>
+      <c r="A13" s="44"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -4599,7 +4655,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="40"/>
+      <c r="A14" s="44"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -4608,7 +4664,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="40"/>
+      <c r="A15" s="44"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -4633,7 +4689,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="40" t="s">
+      <c r="A17" s="44" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -4644,7 +4700,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="40"/>
+      <c r="A18" s="44"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -4653,7 +4709,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="40"/>
+      <c r="A19" s="44"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -4662,7 +4718,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="40"/>
+      <c r="A20" s="44"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -4687,7 +4743,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="40" t="s">
+      <c r="A22" s="44" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -4698,7 +4754,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="40"/>
+      <c r="A23" s="44"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -4707,7 +4763,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="40"/>
+      <c r="A24" s="44"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -4716,7 +4772,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="40"/>
+      <c r="A25" s="44"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -4741,7 +4797,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="40" t="s">
+      <c r="A27" s="44" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -4752,7 +4808,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="40"/>
+      <c r="A28" s="44"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -4761,7 +4817,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="40"/>
+      <c r="A29" s="44"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -4770,7 +4826,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="40"/>
+      <c r="A30" s="44"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -4795,12 +4851,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="36" t="s">
+      <c r="A32" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="36"/>
-      <c r="C32" s="36"/>
-      <c r="D32" s="36"/>
+      <c r="B32" s="40"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="40"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -4811,15 +4867,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="33" t="s">
+      <c r="A33" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="34"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="34"/>
-      <c r="G33" s="35"/>
+      <c r="B33" s="38"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
Finission PCB et documentation
Ajout des modifications finales du PCB et ajout de plusieurs éléments dans la doc.
</commit_message>
<xml_diff>
--- a/jeu_du_moulin_boura/rpt/jeu-du-moulin-bourquenouda-rpt-journal.xlsx
+++ b/jeu_du_moulin_boura/rpt/jeu-du-moulin-bourquenouda-rpt-journal.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bourquenouda01\OneDrive - EDUETATFR\PHIE\jeu_du_moulin_alexandre_bourquenoud\jeu_du_moulin_2025_boura\jeu_du_moulin_boura\rpt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/alexandre_bourquenoud_studentfr_ch/Documents/PHIE/jeu_du_moulin_alexandre_bourquenoud/jeu_du_moulin_2025_boura/jeu_du_moulin_boura/rpt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED970C68-2653-443C-99A4-F9D694477206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{ED970C68-2653-443C-99A4-F9D694477206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A651BEFC-1450-4273-B2E6-B7742EF3AD78}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="71">
   <si>
     <t>Date</t>
   </si>
@@ -313,6 +313,15 @@
       </rPr>
       <t>Je demanderai a M. Egli car il a des meilleur connaissances sur altium.</t>
     </r>
+  </si>
+  <si>
+    <t>j'ai pu ajouter le soldermask au sommet des touches comme voulu grâce à l'aide de M. Egli. En effet, mon erreur était que je n'updatais pas correctement les empreinte.</t>
+  </si>
+  <si>
+    <t>Discussion avec M.Egli au sujet du fonctionnement des touches capacitives et du risque que la matrice LED peut porter à la détection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rédaction de la doc </t>
   </si>
 </sst>
 </file>
@@ -590,18 +599,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -637,6 +634,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1316,19 +1325,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="40" t="s">
+      <c r="D3" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="42" t="s">
+      <c r="E3" s="38" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -1339,11 +1348,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="40"/>
-      <c r="B4" s="40"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="42"/>
+      <c r="A4" s="36"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="38"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -1352,7 +1361,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" s="10" customFormat="1" ht="78.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="39" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -1373,7 +1382,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A6" s="44"/>
+      <c r="A6" s="40"/>
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
@@ -1390,7 +1399,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="44"/>
+      <c r="A7" s="40"/>
       <c r="B7" s="5" t="s">
         <v>22</v>
       </c>
@@ -1409,7 +1418,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="44"/>
+      <c r="A8" s="40"/>
       <c r="B8" s="5" t="s">
         <v>22</v>
       </c>
@@ -1426,7 +1435,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A9" s="44"/>
+      <c r="A9" s="40"/>
       <c r="B9" s="5" t="s">
         <v>22</v>
       </c>
@@ -1443,7 +1452,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" s="10" customFormat="1" ht="78.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="44"/>
+      <c r="A10" s="40"/>
       <c r="B10" s="5" t="s">
         <v>22</v>
       </c>
@@ -1462,7 +1471,7 @@
       <c r="G10" s="14"/>
     </row>
     <row r="11" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A11" s="44"/>
+      <c r="A11" s="40"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -1487,7 +1496,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A13" s="47" t="s">
+      <c r="A13" s="43" t="s">
         <v>5</v>
       </c>
       <c r="B13" s="5" t="s">
@@ -1506,7 +1515,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A14" s="48"/>
+      <c r="A14" s="44"/>
       <c r="B14" s="5" t="s">
         <v>22</v>
       </c>
@@ -1523,7 +1532,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="48"/>
+      <c r="A15" s="44"/>
       <c r="B15" s="5" t="s">
         <v>22</v>
       </c>
@@ -1540,7 +1549,7 @@
       <c r="G15" s="14"/>
     </row>
     <row r="16" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A16" s="48"/>
+      <c r="A16" s="44"/>
       <c r="B16" s="5" t="s">
         <v>22</v>
       </c>
@@ -1557,7 +1566,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A17" s="48"/>
+      <c r="A17" s="44"/>
       <c r="B17" s="5" t="s">
         <v>22</v>
       </c>
@@ -1574,7 +1583,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="48"/>
+      <c r="A18" s="44"/>
       <c r="B18" s="5" t="s">
         <v>22</v>
       </c>
@@ -1591,7 +1600,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A19" s="48"/>
+      <c r="A19" s="44"/>
       <c r="B19" s="5"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -1616,7 +1625,7 @@
       <c r="G20" s="14"/>
     </row>
     <row r="21" spans="1:7" s="10" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
-      <c r="A21" s="43" t="s">
+      <c r="A21" s="39" t="s">
         <v>7</v>
       </c>
       <c r="B21" s="5" t="s">
@@ -1635,7 +1644,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="44"/>
+      <c r="A22" s="40"/>
       <c r="B22" s="5" t="s">
         <v>22</v>
       </c>
@@ -1652,7 +1661,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A23" s="44"/>
+      <c r="A23" s="40"/>
       <c r="B23" s="5" t="s">
         <v>22</v>
       </c>
@@ -1669,7 +1678,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A24" s="44"/>
+      <c r="A24" s="40"/>
       <c r="B24" s="5" t="s">
         <v>22</v>
       </c>
@@ -1686,7 +1695,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A25" s="44"/>
+      <c r="A25" s="40"/>
       <c r="B25" s="5" t="s">
         <v>22</v>
       </c>
@@ -1703,7 +1712,7 @@
       <c r="G25" s="14"/>
     </row>
     <row r="26" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="44"/>
+      <c r="A26" s="40"/>
       <c r="B26" s="5" t="s">
         <v>22</v>
       </c>
@@ -1722,7 +1731,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A27" s="44"/>
+      <c r="A27" s="40"/>
       <c r="B27" s="5" t="s">
         <v>22</v>
       </c>
@@ -1755,7 +1764,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A29" s="43" t="s">
+      <c r="A29" s="39" t="s">
         <v>8</v>
       </c>
       <c r="B29" s="5" t="s">
@@ -1774,7 +1783,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A30" s="44"/>
+      <c r="A30" s="40"/>
       <c r="B30" s="5" t="s">
         <v>22</v>
       </c>
@@ -1793,7 +1802,7 @@
       <c r="G30" s="14"/>
     </row>
     <row r="31" spans="1:7" s="10" customFormat="1" ht="90" x14ac:dyDescent="0.2">
-      <c r="A31" s="44"/>
+      <c r="A31" s="40"/>
       <c r="B31" s="5" t="s">
         <v>22</v>
       </c>
@@ -1812,7 +1821,7 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" s="10" customFormat="1" ht="78.75" x14ac:dyDescent="0.2">
-      <c r="A32" s="44"/>
+      <c r="A32" s="40"/>
       <c r="B32" s="5" t="s">
         <v>22</v>
       </c>
@@ -1829,7 +1838,7 @@
       <c r="G32" s="14"/>
     </row>
     <row r="33" spans="1:7" s="10" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
-      <c r="A33" s="44"/>
+      <c r="A33" s="40"/>
       <c r="B33" s="5" t="s">
         <v>22</v>
       </c>
@@ -1846,7 +1855,7 @@
       <c r="G33" s="14"/>
     </row>
     <row r="34" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A34" s="44"/>
+      <c r="A34" s="40"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
@@ -1873,7 +1882,7 @@
       <c r="G35" s="14"/>
     </row>
     <row r="36" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A36" s="43" t="s">
+      <c r="A36" s="39" t="s">
         <v>9</v>
       </c>
       <c r="B36" s="5" t="s">
@@ -1892,7 +1901,7 @@
       <c r="G36" s="14"/>
     </row>
     <row r="37" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A37" s="44"/>
+      <c r="A37" s="40"/>
       <c r="B37" s="5" t="s">
         <v>22</v>
       </c>
@@ -1907,7 +1916,7 @@
       <c r="G37" s="14"/>
     </row>
     <row r="38" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A38" s="44"/>
+      <c r="A38" s="40"/>
       <c r="B38" s="5" t="s">
         <v>22</v>
       </c>
@@ -1926,7 +1935,7 @@
       <c r="G38" s="14"/>
     </row>
     <row r="39" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A39" s="44"/>
+      <c r="A39" s="40"/>
       <c r="B39" s="5" t="s">
         <v>22</v>
       </c>
@@ -1945,7 +1954,7 @@
       <c r="G39" s="14"/>
     </row>
     <row r="40" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A40" s="44"/>
+      <c r="A40" s="40"/>
       <c r="B40" s="5"/>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
@@ -1970,12 +1979,12 @@
       <c r="G41" s="14"/>
     </row>
     <row r="42" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="42" t="s">
+      <c r="A42" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="B42" s="45"/>
-      <c r="C42" s="45"/>
-      <c r="D42" s="46"/>
+      <c r="B42" s="41"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="42"/>
       <c r="E42" s="17"/>
       <c r="F42" s="17" t="s">
         <v>12</v>
@@ -1986,36 +1995,36 @@
       </c>
     </row>
     <row r="43" spans="1:7" s="10" customFormat="1" ht="82.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="37" t="s">
+      <c r="A43" s="33" t="s">
         <v>62</v>
       </c>
-      <c r="B43" s="38"/>
-      <c r="C43" s="38"/>
-      <c r="D43" s="38"/>
-      <c r="E43" s="38"/>
-      <c r="F43" s="38"/>
-      <c r="G43" s="39"/>
+      <c r="B43" s="34"/>
+      <c r="C43" s="34"/>
+      <c r="D43" s="34"/>
+      <c r="E43" s="34"/>
+      <c r="F43" s="34"/>
+      <c r="G43" s="35"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="34"/>
-      <c r="B46" s="34"/>
-      <c r="C46" s="36"/>
-      <c r="D46" s="34"/>
-      <c r="E46" s="34"/>
+      <c r="A46" s="45"/>
+      <c r="B46" s="45"/>
+      <c r="C46" s="46"/>
+      <c r="D46" s="45"/>
+      <c r="E46" s="45"/>
       <c r="F46" s="23"/>
       <c r="G46" s="23"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="34"/>
-      <c r="B47" s="34"/>
-      <c r="C47" s="36"/>
-      <c r="D47" s="34"/>
-      <c r="E47" s="34"/>
+      <c r="A47" s="45"/>
+      <c r="B47" s="45"/>
+      <c r="C47" s="46"/>
+      <c r="D47" s="45"/>
+      <c r="E47" s="45"/>
       <c r="F47" s="23"/>
       <c r="G47" s="23"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="33"/>
+      <c r="A48" s="47"/>
       <c r="B48" s="25"/>
       <c r="C48" s="25"/>
       <c r="D48" s="25"/>
@@ -2024,7 +2033,7 @@
       <c r="G48" s="10"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="33"/>
+      <c r="A49" s="47"/>
       <c r="B49" s="25"/>
       <c r="C49" s="25"/>
       <c r="D49" s="25"/>
@@ -2033,7 +2042,7 @@
       <c r="G49" s="10"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="33"/>
+      <c r="A50" s="47"/>
       <c r="B50" s="25"/>
       <c r="C50" s="25"/>
       <c r="D50" s="25"/>
@@ -2042,7 +2051,7 @@
       <c r="G50" s="10"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="33"/>
+      <c r="A51" s="47"/>
       <c r="B51" s="25"/>
       <c r="C51" s="25"/>
       <c r="D51" s="25"/>
@@ -2051,7 +2060,7 @@
       <c r="G51" s="10"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="33"/>
+      <c r="A52" s="47"/>
       <c r="B52" s="25"/>
       <c r="C52" s="25"/>
       <c r="D52" s="25"/>
@@ -2060,7 +2069,7 @@
       <c r="G52" s="10"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="33"/>
+      <c r="A53" s="47"/>
       <c r="B53" s="25"/>
       <c r="C53" s="25"/>
       <c r="D53" s="25"/>
@@ -2078,7 +2087,7 @@
       <c r="G54" s="10"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="33"/>
+      <c r="A55" s="47"/>
       <c r="B55" s="25"/>
       <c r="C55" s="25"/>
       <c r="D55" s="25"/>
@@ -2087,7 +2096,7 @@
       <c r="G55" s="10"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="33"/>
+      <c r="A56" s="47"/>
       <c r="B56" s="25"/>
       <c r="C56" s="25"/>
       <c r="D56" s="25"/>
@@ -2096,7 +2105,7 @@
       <c r="G56" s="10"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="33"/>
+      <c r="A57" s="47"/>
       <c r="B57" s="25"/>
       <c r="C57" s="25"/>
       <c r="D57" s="25"/>
@@ -2105,7 +2114,7 @@
       <c r="G57" s="10"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="33"/>
+      <c r="A58" s="47"/>
       <c r="B58" s="25"/>
       <c r="C58" s="25"/>
       <c r="D58" s="25"/>
@@ -2123,7 +2132,7 @@
       <c r="G59" s="10"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="33"/>
+      <c r="A60" s="47"/>
       <c r="B60" s="25"/>
       <c r="C60" s="25"/>
       <c r="D60" s="25"/>
@@ -2132,7 +2141,7 @@
       <c r="G60" s="10"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="33"/>
+      <c r="A61" s="47"/>
       <c r="B61" s="25"/>
       <c r="C61" s="25"/>
       <c r="D61" s="25"/>
@@ -2141,7 +2150,7 @@
       <c r="G61" s="10"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="33"/>
+      <c r="A62" s="47"/>
       <c r="B62" s="25"/>
       <c r="C62" s="25"/>
       <c r="D62" s="25"/>
@@ -2150,7 +2159,7 @@
       <c r="G62" s="10"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="33"/>
+      <c r="A63" s="47"/>
       <c r="B63" s="25"/>
       <c r="C63" s="25"/>
       <c r="D63" s="25"/>
@@ -2168,7 +2177,7 @@
       <c r="G64" s="10"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" s="33"/>
+      <c r="A65" s="47"/>
       <c r="B65" s="25"/>
       <c r="C65" s="25"/>
       <c r="D65" s="25"/>
@@ -2177,7 +2186,7 @@
       <c r="G65" s="10"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" s="33"/>
+      <c r="A66" s="47"/>
       <c r="B66" s="25"/>
       <c r="C66" s="25"/>
       <c r="D66" s="25"/>
@@ -2186,7 +2195,7 @@
       <c r="G66" s="10"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" s="33"/>
+      <c r="A67" s="47"/>
       <c r="B67" s="25"/>
       <c r="C67" s="25"/>
       <c r="D67" s="25"/>
@@ -2195,7 +2204,7 @@
       <c r="G67" s="10"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" s="33"/>
+      <c r="A68" s="47"/>
       <c r="B68" s="25"/>
       <c r="C68" s="25"/>
       <c r="D68" s="25"/>
@@ -2213,7 +2222,7 @@
       <c r="G69" s="10"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" s="33"/>
+      <c r="A70" s="47"/>
       <c r="B70" s="25"/>
       <c r="C70" s="25"/>
       <c r="D70" s="25"/>
@@ -2222,7 +2231,7 @@
       <c r="G70" s="10"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" s="33"/>
+      <c r="A71" s="47"/>
       <c r="B71" s="25"/>
       <c r="C71" s="25"/>
       <c r="D71" s="25"/>
@@ -2231,7 +2240,7 @@
       <c r="G71" s="10"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" s="33"/>
+      <c r="A72" s="47"/>
       <c r="B72" s="25"/>
       <c r="C72" s="25"/>
       <c r="D72" s="25"/>
@@ -2240,7 +2249,7 @@
       <c r="G72" s="10"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A73" s="33"/>
+      <c r="A73" s="47"/>
       <c r="B73" s="25"/>
       <c r="C73" s="25"/>
       <c r="D73" s="25"/>
@@ -2258,25 +2267,37 @@
       <c r="G74" s="10"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" s="34"/>
-      <c r="B75" s="34"/>
-      <c r="C75" s="34"/>
-      <c r="D75" s="34"/>
+      <c r="A75" s="45"/>
+      <c r="B75" s="45"/>
+      <c r="C75" s="45"/>
+      <c r="D75" s="45"/>
       <c r="E75" s="27"/>
       <c r="F75" s="27"/>
       <c r="G75" s="28"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" s="35"/>
-      <c r="B76" s="35"/>
-      <c r="C76" s="35"/>
-      <c r="D76" s="35"/>
-      <c r="E76" s="35"/>
-      <c r="F76" s="35"/>
-      <c r="G76" s="35"/>
+      <c r="A76" s="48"/>
+      <c r="B76" s="48"/>
+      <c r="C76" s="48"/>
+      <c r="D76" s="48"/>
+      <c r="E76" s="48"/>
+      <c r="F76" s="48"/>
+      <c r="G76" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A48:A53"/>
+    <mergeCell ref="A75:D75"/>
+    <mergeCell ref="A76:G76"/>
+    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="A60:A63"/>
+    <mergeCell ref="A65:A68"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="E46:E47"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
@@ -2289,18 +2310,6 @@
     <mergeCell ref="A36:A40"/>
     <mergeCell ref="A42:D42"/>
     <mergeCell ref="A13:A19"/>
-    <mergeCell ref="A46:A47"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="E46:E47"/>
-    <mergeCell ref="A48:A53"/>
-    <mergeCell ref="A75:D75"/>
-    <mergeCell ref="A76:G76"/>
-    <mergeCell ref="A55:A58"/>
-    <mergeCell ref="A60:A63"/>
-    <mergeCell ref="A65:A68"/>
-    <mergeCell ref="A70:A73"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F16 F20:F41">
     <cfRule type="containsText" dxfId="31" priority="1" operator="containsText" text="Terminé">
@@ -2341,7 +2350,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" style="1" customWidth="1"/>
@@ -2381,19 +2390,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="40" t="s">
+      <c r="D3" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="42" t="s">
+      <c r="E3" s="38" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -2404,11 +2413,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="40"/>
-      <c r="B4" s="40"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="42"/>
+      <c r="A4" s="36"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="38"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -2417,7 +2426,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="39" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -2436,7 +2445,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A6" s="44"/>
+      <c r="A6" s="40"/>
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
@@ -2453,7 +2462,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" s="10" customFormat="1" ht="90" x14ac:dyDescent="0.2">
-      <c r="A7" s="44"/>
+      <c r="A7" s="40"/>
       <c r="B7" s="5" t="s">
         <v>22</v>
       </c>
@@ -2472,7 +2481,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="44"/>
+      <c r="A8" s="40"/>
       <c r="B8" s="5" t="s">
         <v>22</v>
       </c>
@@ -2489,7 +2498,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="44"/>
+      <c r="A9" s="40"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -2498,7 +2507,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="44"/>
+      <c r="A10" s="40"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -2522,83 +2531,115 @@
       </c>
       <c r="G11" s="14"/>
     </row>
-    <row r="12" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A12" s="44" t="s">
+    <row r="12" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
+      <c r="A12" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
+      <c r="B12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="E12" s="4"/>
-      <c r="F12" s="6"/>
+      <c r="F12" s="13">
+        <v>0.2</v>
+      </c>
       <c r="G12" s="14"/>
     </row>
-    <row r="13" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A13" s="44"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
+    <row r="13" spans="1:7" s="10" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
+      <c r="A13" s="40"/>
+      <c r="B13" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>68</v>
+      </c>
       <c r="E13" s="4"/>
-      <c r="F13" s="6"/>
+      <c r="F13" s="6">
+        <v>3.3</v>
+      </c>
       <c r="G13" s="14"/>
     </row>
-    <row r="14" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A14" s="44"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
+    <row r="14" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
+      <c r="A14" s="40"/>
+      <c r="B14" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>70</v>
+      </c>
       <c r="E14" s="4"/>
-      <c r="F14" s="6"/>
+      <c r="F14" s="6">
+        <v>3.3</v>
+      </c>
       <c r="G14" s="14"/>
     </row>
-    <row r="15" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="44"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
+    <row r="15" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
+      <c r="A15" s="40"/>
+      <c r="B15" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>69</v>
+      </c>
       <c r="E15" s="4"/>
-      <c r="F15" s="6"/>
+      <c r="F15" s="6">
+        <v>0.2</v>
+      </c>
       <c r="G15" s="14"/>
     </row>
-    <row r="16" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A16" s="31">
+    <row r="16" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="40"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="14"/>
+    </row>
+    <row r="17" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A17" s="31">
         <v>45797</v>
       </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="17" t="s">
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="F16" s="18">
-        <f>SUM(F12:F15)</f>
-        <v>0</v>
-      </c>
-      <c r="G16" s="14"/>
-    </row>
-    <row r="17" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A17" s="44" t="s">
+      <c r="F17" s="18">
+        <f>SUM(F12:F16)</f>
         <v>7</v>
       </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="6"/>
       <c r="G17" s="14"/>
-      <c r="J17" s="32"/>
     </row>
     <row r="18" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A18" s="44"/>
+      <c r="A18" s="40" t="s">
+        <v>7</v>
+      </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="F18" s="6"/>
       <c r="G18" s="14"/>
+      <c r="J18" s="32"/>
     </row>
     <row r="19" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A19" s="44"/>
+      <c r="A19" s="40"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -2606,8 +2647,8 @@
       <c r="F19" s="6"/>
       <c r="G19" s="14"/>
     </row>
-    <row r="20" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="44"/>
+    <row r="20" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A20" s="40"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -2615,45 +2656,44 @@
       <c r="F20" s="6"/>
       <c r="G20" s="14"/>
     </row>
-    <row r="21" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A21" s="31">
+    <row r="21" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="40"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="14"/>
+    </row>
+    <row r="22" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A22" s="31">
         <v>45798</v>
       </c>
-      <c r="B21" s="16"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="17" t="s">
+      <c r="B22" s="16"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="F21" s="18">
-        <f>SUM(F17:F20)</f>
+      <c r="F22" s="18">
+        <f>SUM(F18:F21)</f>
         <v>0</v>
       </c>
-      <c r="G21" s="14"/>
-    </row>
-    <row r="22" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A22" s="44" t="s">
+      <c r="G22" s="14"/>
+    </row>
+    <row r="23" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A23" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="14"/>
-    </row>
-    <row r="23" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A23" s="44"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
       <c r="F23" s="6"/>
       <c r="G23" s="14"/>
-      <c r="J23" s="32"/>
     </row>
     <row r="24" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A24" s="44"/>
+      <c r="A24" s="40"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -2662,44 +2702,45 @@
       <c r="G24" s="14"/>
       <c r="J24" s="32"/>
     </row>
-    <row r="25" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="44"/>
+    <row r="25" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A25" s="40"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
       <c r="F25" s="6"/>
       <c r="G25" s="14"/>
-    </row>
-    <row r="26" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="31">
+      <c r="J25" s="32"/>
+    </row>
+    <row r="26" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="40"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="14"/>
+    </row>
+    <row r="27" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A27" s="31">
         <v>45799</v>
       </c>
-      <c r="B26" s="16"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="17" t="s">
+      <c r="B27" s="16"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="F26" s="18">
-        <f>SUM(F22:F25)</f>
+      <c r="F27" s="18">
+        <f>SUM(F23:F26)</f>
         <v>0</v>
       </c>
-      <c r="G26" s="14"/>
-    </row>
-    <row r="27" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A27" s="44" t="s">
+      <c r="G27" s="14"/>
+    </row>
+    <row r="28" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A28" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="14"/>
-    </row>
-    <row r="28" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A28" s="44"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -2708,7 +2749,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A29" s="44"/>
+      <c r="A29" s="40"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -2716,8 +2757,8 @@
       <c r="F29" s="6"/>
       <c r="G29" s="14"/>
     </row>
-    <row r="30" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="44"/>
+    <row r="30" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A30" s="40"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -2726,64 +2767,73 @@
       <c r="G30" s="14"/>
     </row>
     <row r="31" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="31">
+      <c r="A31" s="40"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="14"/>
+    </row>
+    <row r="32" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="31">
         <v>45800</v>
       </c>
-      <c r="B31" s="19"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="20" t="s">
+      <c r="B32" s="19"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="F31" s="21">
-        <f>SUM(F27:F30)</f>
+      <c r="F32" s="21">
+        <f>SUM(F28:F31)</f>
         <v>0</v>
       </c>
-      <c r="G31" s="14"/>
-    </row>
-    <row r="32" spans="1:10" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="40" t="s">
+      <c r="G32" s="14"/>
+    </row>
+    <row r="33" spans="1:7" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="40"/>
-      <c r="C32" s="40"/>
-      <c r="D32" s="40"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17" t="s">
+      <c r="B33" s="36"/>
+      <c r="C33" s="36"/>
+      <c r="D33" s="36"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="G32" s="22">
-        <f>F11+F16+F21+F26+F31</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="37" t="s">
+      <c r="G33" s="22">
+        <f>F11+F17+F22+F27+F32</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="38"/>
-      <c r="C33" s="38"/>
-      <c r="D33" s="38"/>
-      <c r="E33" s="38"/>
-      <c r="F33" s="38"/>
-      <c r="G33" s="39"/>
+      <c r="B34" s="34"/>
+      <c r="C34" s="34"/>
+      <c r="D34" s="34"/>
+      <c r="E34" s="34"/>
+      <c r="F34" s="34"/>
+      <c r="G34" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A34:G34"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="A5:A10"/>
-    <mergeCell ref="A12:A15"/>
-    <mergeCell ref="A17:A20"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A27:A30"/>
-    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A12:A16"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A23:A26"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="A33:D33"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F31">
+  <conditionalFormatting sqref="F5:F32">
     <cfRule type="containsText" dxfId="23" priority="1" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",F5)))</formula>
     </cfRule>
@@ -2791,12 +2841,12 @@
       <formula>NOT(ISERROR(SEARCH("En cours",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G32">
+  <conditionalFormatting sqref="G33">
     <cfRule type="containsText" dxfId="21" priority="3" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",G32)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",G33)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="20" priority="4" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",G32)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",G33)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2841,19 +2891,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="40" t="s">
+      <c r="D3" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="42" t="s">
+      <c r="E3" s="38" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -2864,11 +2914,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="40"/>
-      <c r="B4" s="40"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="42"/>
+      <c r="A4" s="36"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="38"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -2877,7 +2927,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="39" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -2888,7 +2938,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="44"/>
+      <c r="A6" s="40"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -2897,7 +2947,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="44"/>
+      <c r="A7" s="40"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -2906,7 +2956,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="44"/>
+      <c r="A8" s="40"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -2915,7 +2965,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="44"/>
+      <c r="A9" s="40"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -2924,7 +2974,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="44"/>
+      <c r="A10" s="40"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -2949,7 +2999,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="44" t="s">
+      <c r="A12" s="40" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -2960,7 +3010,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="44"/>
+      <c r="A13" s="40"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -2969,7 +3019,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="44"/>
+      <c r="A14" s="40"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -2978,7 +3028,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="44"/>
+      <c r="A15" s="40"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -3003,7 +3053,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="44" t="s">
+      <c r="A17" s="40" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -3014,7 +3064,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="44"/>
+      <c r="A18" s="40"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -3023,7 +3073,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="44"/>
+      <c r="A19" s="40"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -3032,7 +3082,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="44"/>
+      <c r="A20" s="40"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -3057,7 +3107,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="44" t="s">
+      <c r="A22" s="40" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -3068,7 +3118,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="44"/>
+      <c r="A23" s="40"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -3077,7 +3127,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="44"/>
+      <c r="A24" s="40"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -3086,7 +3136,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="44"/>
+      <c r="A25" s="40"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -3111,7 +3161,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="44" t="s">
+      <c r="A27" s="40" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -3122,7 +3172,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="44"/>
+      <c r="A28" s="40"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -3131,7 +3181,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="44"/>
+      <c r="A29" s="40"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -3140,7 +3190,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="44"/>
+      <c r="A30" s="40"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -3165,12 +3215,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="40" t="s">
+      <c r="A32" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="40"/>
-      <c r="C32" s="40"/>
-      <c r="D32" s="40"/>
+      <c r="B32" s="36"/>
+      <c r="C32" s="36"/>
+      <c r="D32" s="36"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -3181,18 +3231,23 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="37" t="s">
+      <c r="A33" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="38"/>
-      <c r="C33" s="38"/>
-      <c r="D33" s="38"/>
-      <c r="E33" s="38"/>
-      <c r="F33" s="38"/>
-      <c r="G33" s="39"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="34"/>
+      <c r="E33" s="34"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A5:A10"/>
@@ -3200,11 +3255,6 @@
     <mergeCell ref="A17:A20"/>
     <mergeCell ref="A22:A25"/>
     <mergeCell ref="A27:A30"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F31">
     <cfRule type="containsText" dxfId="19" priority="1" operator="containsText" text="Terminé">
@@ -3262,19 +3312,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="40" t="s">
+      <c r="D3" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="42" t="s">
+      <c r="E3" s="38" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -3285,11 +3335,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="40"/>
-      <c r="B4" s="40"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="42"/>
+      <c r="A4" s="36"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="38"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -3298,7 +3348,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="39" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -3309,7 +3359,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="44"/>
+      <c r="A6" s="40"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -3318,7 +3368,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="44"/>
+      <c r="A7" s="40"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -3327,7 +3377,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="44"/>
+      <c r="A8" s="40"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -3336,7 +3386,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="44"/>
+      <c r="A9" s="40"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -3345,7 +3395,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="44"/>
+      <c r="A10" s="40"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -3370,7 +3420,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="44" t="s">
+      <c r="A12" s="40" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -3381,7 +3431,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="44"/>
+      <c r="A13" s="40"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -3390,7 +3440,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="44"/>
+      <c r="A14" s="40"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -3399,7 +3449,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="44"/>
+      <c r="A15" s="40"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -3424,7 +3474,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="44" t="s">
+      <c r="A17" s="40" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -3435,7 +3485,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="44"/>
+      <c r="A18" s="40"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -3444,7 +3494,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="44"/>
+      <c r="A19" s="40"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -3453,7 +3503,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="44"/>
+      <c r="A20" s="40"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -3478,7 +3528,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="44" t="s">
+      <c r="A22" s="40" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -3489,7 +3539,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="44"/>
+      <c r="A23" s="40"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -3498,7 +3548,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="44"/>
+      <c r="A24" s="40"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -3507,7 +3557,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="44"/>
+      <c r="A25" s="40"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -3532,7 +3582,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="44" t="s">
+      <c r="A27" s="40" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -3543,7 +3593,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="44"/>
+      <c r="A28" s="40"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -3552,7 +3602,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="44"/>
+      <c r="A29" s="40"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -3561,7 +3611,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="44"/>
+      <c r="A30" s="40"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -3586,12 +3636,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="40" t="s">
+      <c r="A32" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="40"/>
-      <c r="C32" s="40"/>
-      <c r="D32" s="40"/>
+      <c r="B32" s="36"/>
+      <c r="C32" s="36"/>
+      <c r="D32" s="36"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -3602,18 +3652,23 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="37" t="s">
+      <c r="A33" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="38"/>
-      <c r="C33" s="38"/>
-      <c r="D33" s="38"/>
-      <c r="E33" s="38"/>
-      <c r="F33" s="38"/>
-      <c r="G33" s="39"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="34"/>
+      <c r="E33" s="34"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A5:A10"/>
@@ -3621,11 +3676,6 @@
     <mergeCell ref="A17:A20"/>
     <mergeCell ref="A22:A25"/>
     <mergeCell ref="A27:A30"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F31">
     <cfRule type="containsText" dxfId="15" priority="1" operator="containsText" text="Terminé">
@@ -3683,19 +3733,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="40" t="s">
+      <c r="D3" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="42" t="s">
+      <c r="E3" s="38" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -3706,11 +3756,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="40"/>
-      <c r="B4" s="40"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="42"/>
+      <c r="A4" s="36"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="38"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -3719,7 +3769,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="39" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -3730,7 +3780,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="44"/>
+      <c r="A6" s="40"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -3739,7 +3789,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="44"/>
+      <c r="A7" s="40"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -3748,7 +3798,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="44"/>
+      <c r="A8" s="40"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -3757,7 +3807,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="44"/>
+      <c r="A9" s="40"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -3766,7 +3816,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="44"/>
+      <c r="A10" s="40"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -3791,7 +3841,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="44" t="s">
+      <c r="A12" s="40" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -3802,7 +3852,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="44"/>
+      <c r="A13" s="40"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -3811,7 +3861,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="44"/>
+      <c r="A14" s="40"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -3820,7 +3870,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="44"/>
+      <c r="A15" s="40"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -3845,7 +3895,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="44" t="s">
+      <c r="A17" s="40" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -3856,7 +3906,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="44"/>
+      <c r="A18" s="40"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -3865,7 +3915,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="44"/>
+      <c r="A19" s="40"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -3874,7 +3924,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="44"/>
+      <c r="A20" s="40"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -3899,7 +3949,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="44" t="s">
+      <c r="A22" s="40" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -3910,7 +3960,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="44"/>
+      <c r="A23" s="40"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -3919,7 +3969,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="44"/>
+      <c r="A24" s="40"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -3928,7 +3978,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="44"/>
+      <c r="A25" s="40"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -3953,7 +4003,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="44" t="s">
+      <c r="A27" s="40" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -3964,7 +4014,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="44"/>
+      <c r="A28" s="40"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -3973,7 +4023,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="44"/>
+      <c r="A29" s="40"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -3982,7 +4032,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="44"/>
+      <c r="A30" s="40"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -4007,12 +4057,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="40" t="s">
+      <c r="A32" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="40"/>
-      <c r="C32" s="40"/>
-      <c r="D32" s="40"/>
+      <c r="B32" s="36"/>
+      <c r="C32" s="36"/>
+      <c r="D32" s="36"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -4023,15 +4073,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="37" t="s">
+      <c r="A33" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="38"/>
-      <c r="C33" s="38"/>
-      <c r="D33" s="38"/>
-      <c r="E33" s="38"/>
-      <c r="F33" s="38"/>
-      <c r="G33" s="39"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="34"/>
+      <c r="E33" s="34"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -4106,19 +4156,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="40" t="s">
+      <c r="D3" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="42" t="s">
+      <c r="E3" s="38" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -4129,11 +4179,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="40"/>
-      <c r="B4" s="40"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="42"/>
+      <c r="A4" s="36"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="38"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -4142,7 +4192,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="39" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -4153,7 +4203,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="44"/>
+      <c r="A6" s="40"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -4162,7 +4212,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="44"/>
+      <c r="A7" s="40"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -4171,7 +4221,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="44"/>
+      <c r="A8" s="40"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -4180,7 +4230,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="44"/>
+      <c r="A9" s="40"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -4189,7 +4239,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="44"/>
+      <c r="A10" s="40"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -4214,7 +4264,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="44" t="s">
+      <c r="A12" s="40" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -4225,7 +4275,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="44"/>
+      <c r="A13" s="40"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -4234,7 +4284,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="44"/>
+      <c r="A14" s="40"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -4243,7 +4293,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="44"/>
+      <c r="A15" s="40"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -4268,7 +4318,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="44" t="s">
+      <c r="A17" s="40" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -4279,7 +4329,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="44"/>
+      <c r="A18" s="40"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -4288,7 +4338,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="44"/>
+      <c r="A19" s="40"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -4297,7 +4347,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="44"/>
+      <c r="A20" s="40"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -4322,7 +4372,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="44" t="s">
+      <c r="A22" s="40" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -4333,7 +4383,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="44"/>
+      <c r="A23" s="40"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -4342,7 +4392,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="44"/>
+      <c r="A24" s="40"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -4351,7 +4401,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="44"/>
+      <c r="A25" s="40"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -4376,7 +4426,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="44" t="s">
+      <c r="A27" s="40" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -4387,7 +4437,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="44"/>
+      <c r="A28" s="40"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -4396,7 +4446,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="44"/>
+      <c r="A29" s="40"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -4405,7 +4455,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="44"/>
+      <c r="A30" s="40"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -4430,12 +4480,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="40" t="s">
+      <c r="A32" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="40"/>
-      <c r="C32" s="40"/>
-      <c r="D32" s="40"/>
+      <c r="B32" s="36"/>
+      <c r="C32" s="36"/>
+      <c r="D32" s="36"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -4446,15 +4496,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="37" t="s">
+      <c r="A33" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="38"/>
-      <c r="C33" s="38"/>
-      <c r="D33" s="38"/>
-      <c r="E33" s="38"/>
-      <c r="F33" s="38"/>
-      <c r="G33" s="39"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="34"/>
+      <c r="E33" s="34"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -4527,19 +4577,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="40" t="s">
+      <c r="D3" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="42" t="s">
+      <c r="E3" s="38" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -4550,11 +4600,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="40"/>
-      <c r="B4" s="40"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="42"/>
+      <c r="A4" s="36"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="38"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -4563,7 +4613,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="39" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -4574,7 +4624,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="44"/>
+      <c r="A6" s="40"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -4583,7 +4633,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="44"/>
+      <c r="A7" s="40"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -4592,7 +4642,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="44"/>
+      <c r="A8" s="40"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -4601,7 +4651,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="44"/>
+      <c r="A9" s="40"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -4610,7 +4660,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="44"/>
+      <c r="A10" s="40"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -4635,7 +4685,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="44" t="s">
+      <c r="A12" s="40" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -4646,7 +4696,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="44"/>
+      <c r="A13" s="40"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -4655,7 +4705,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="44"/>
+      <c r="A14" s="40"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -4664,7 +4714,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="44"/>
+      <c r="A15" s="40"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -4689,7 +4739,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="44" t="s">
+      <c r="A17" s="40" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -4700,7 +4750,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="44"/>
+      <c r="A18" s="40"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -4709,7 +4759,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="44"/>
+      <c r="A19" s="40"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -4718,7 +4768,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="44"/>
+      <c r="A20" s="40"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -4743,7 +4793,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="44" t="s">
+      <c r="A22" s="40" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -4754,7 +4804,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="44"/>
+      <c r="A23" s="40"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -4763,7 +4813,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="44"/>
+      <c r="A24" s="40"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -4772,7 +4822,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="44"/>
+      <c r="A25" s="40"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -4797,7 +4847,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="44" t="s">
+      <c r="A27" s="40" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -4808,7 +4858,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="44"/>
+      <c r="A28" s="40"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -4817,7 +4867,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="44"/>
+      <c r="A29" s="40"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -4826,7 +4876,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="44"/>
+      <c r="A30" s="40"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -4851,12 +4901,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="40" t="s">
+      <c r="A32" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="40"/>
-      <c r="C32" s="40"/>
-      <c r="D32" s="40"/>
+      <c r="B32" s="36"/>
+      <c r="C32" s="36"/>
+      <c r="D32" s="36"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -4867,15 +4917,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="37" t="s">
+      <c r="A33" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="38"/>
-      <c r="C33" s="38"/>
-      <c r="D33" s="38"/>
-      <c r="E33" s="38"/>
-      <c r="F33" s="38"/>
-      <c r="G33" s="39"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="34"/>
+      <c r="E33" s="34"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
Modification finales du PCB et création des Gerber
J'ai fini les dernier changements de routage pour les LEDs en dessous des touches et la convenance à la classe 6C de Eurocircuit puis j'ai fini les gerbers
</commit_message>
<xml_diff>
--- a/jeu_du_moulin_boura/rpt/jeu-du-moulin-bourquenouda-rpt-journal.xlsx
+++ b/jeu_du_moulin_boura/rpt/jeu-du-moulin-bourquenouda-rpt-journal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/alexandre_bourquenoud_studentfr_ch/Documents/PHIE/jeu_du_moulin_alexandre_bourquenoud/jeu_du_moulin_2025_boura/jeu_du_moulin_boura/rpt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="149" documentId="13_ncr:1_{ED970C68-2653-443C-99A4-F9D694477206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07AA70EE-31AD-430E-9B3C-591C045B6107}"/>
+  <xr:revisionPtr revIDLastSave="154" documentId="13_ncr:1_{ED970C68-2653-443C-99A4-F9D694477206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D33F6F5-A8DD-402B-9B04-39EFC4D80797}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="75">
   <si>
     <t>Date</t>
   </si>
@@ -331,6 +331,9 @@
   </si>
   <si>
     <t>création des Gerber et vérification sur eurocircuit de la classe et validité du circuit.</t>
+  </si>
+  <si>
+    <t>finission des dernier détails du pcb par example amélioration du routage des pistes et création des Gerber et vérification sur eurocircuit de la classe et validité du circuit.</t>
   </si>
 </sst>
 </file>
@@ -617,18 +620,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -664,6 +655,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1347,19 +1350,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="C3" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="43" t="s">
+      <c r="D3" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="45" t="s">
+      <c r="E3" s="41" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -1370,11 +1373,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="43"/>
-      <c r="B4" s="43"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="45"/>
+      <c r="A4" s="39"/>
+      <c r="B4" s="39"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -1383,7 +1386,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" s="10" customFormat="1" ht="78.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="42" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -1404,7 +1407,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A6" s="47"/>
+      <c r="A6" s="43"/>
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
@@ -1421,7 +1424,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="47"/>
+      <c r="A7" s="43"/>
       <c r="B7" s="5" t="s">
         <v>22</v>
       </c>
@@ -1438,7 +1441,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="47"/>
+      <c r="A8" s="43"/>
       <c r="B8" s="5" t="s">
         <v>22</v>
       </c>
@@ -1455,7 +1458,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A9" s="47"/>
+      <c r="A9" s="43"/>
       <c r="B9" s="5" t="s">
         <v>22</v>
       </c>
@@ -1472,7 +1475,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" s="10" customFormat="1" ht="78.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="47"/>
+      <c r="A10" s="43"/>
       <c r="B10" s="5" t="s">
         <v>22</v>
       </c>
@@ -1491,7 +1494,7 @@
       <c r="G10" s="14"/>
     </row>
     <row r="11" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A11" s="47"/>
+      <c r="A11" s="43"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -1516,7 +1519,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A13" s="50" t="s">
+      <c r="A13" s="46" t="s">
         <v>5</v>
       </c>
       <c r="B13" s="5" t="s">
@@ -1535,7 +1538,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A14" s="51"/>
+      <c r="A14" s="47"/>
       <c r="B14" s="5" t="s">
         <v>22</v>
       </c>
@@ -1552,7 +1555,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="51"/>
+      <c r="A15" s="47"/>
       <c r="B15" s="5" t="s">
         <v>22</v>
       </c>
@@ -1569,7 +1572,7 @@
       <c r="G15" s="14"/>
     </row>
     <row r="16" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A16" s="51"/>
+      <c r="A16" s="47"/>
       <c r="B16" s="5" t="s">
         <v>22</v>
       </c>
@@ -1586,7 +1589,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A17" s="51"/>
+      <c r="A17" s="47"/>
       <c r="B17" s="5" t="s">
         <v>22</v>
       </c>
@@ -1603,7 +1606,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="51"/>
+      <c r="A18" s="47"/>
       <c r="B18" s="5" t="s">
         <v>22</v>
       </c>
@@ -1620,7 +1623,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A19" s="51"/>
+      <c r="A19" s="47"/>
       <c r="B19" s="5"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -1645,7 +1648,7 @@
       <c r="G20" s="14"/>
     </row>
     <row r="21" spans="1:7" s="10" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
-      <c r="A21" s="46" t="s">
+      <c r="A21" s="42" t="s">
         <v>7</v>
       </c>
       <c r="B21" s="5" t="s">
@@ -1664,7 +1667,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="47"/>
+      <c r="A22" s="43"/>
       <c r="B22" s="5" t="s">
         <v>22</v>
       </c>
@@ -1681,7 +1684,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A23" s="47"/>
+      <c r="A23" s="43"/>
       <c r="B23" s="5" t="s">
         <v>22</v>
       </c>
@@ -1698,7 +1701,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A24" s="47"/>
+      <c r="A24" s="43"/>
       <c r="B24" s="5" t="s">
         <v>22</v>
       </c>
@@ -1715,7 +1718,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A25" s="47"/>
+      <c r="A25" s="43"/>
       <c r="B25" s="5" t="s">
         <v>22</v>
       </c>
@@ -1732,7 +1735,7 @@
       <c r="G25" s="14"/>
     </row>
     <row r="26" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="47"/>
+      <c r="A26" s="43"/>
       <c r="B26" s="5" t="s">
         <v>22</v>
       </c>
@@ -1751,7 +1754,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A27" s="47"/>
+      <c r="A27" s="43"/>
       <c r="B27" s="5" t="s">
         <v>22</v>
       </c>
@@ -1784,7 +1787,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A29" s="46" t="s">
+      <c r="A29" s="42" t="s">
         <v>8</v>
       </c>
       <c r="B29" s="5" t="s">
@@ -1803,7 +1806,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A30" s="47"/>
+      <c r="A30" s="43"/>
       <c r="B30" s="5" t="s">
         <v>22</v>
       </c>
@@ -1822,7 +1825,7 @@
       <c r="G30" s="14"/>
     </row>
     <row r="31" spans="1:7" s="10" customFormat="1" ht="90" x14ac:dyDescent="0.2">
-      <c r="A31" s="47"/>
+      <c r="A31" s="43"/>
       <c r="B31" s="5" t="s">
         <v>22</v>
       </c>
@@ -1841,7 +1844,7 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" s="10" customFormat="1" ht="78.75" x14ac:dyDescent="0.2">
-      <c r="A32" s="47"/>
+      <c r="A32" s="43"/>
       <c r="B32" s="5" t="s">
         <v>22</v>
       </c>
@@ -1858,7 +1861,7 @@
       <c r="G32" s="14"/>
     </row>
     <row r="33" spans="1:7" s="10" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
-      <c r="A33" s="47"/>
+      <c r="A33" s="43"/>
       <c r="B33" s="5" t="s">
         <v>22</v>
       </c>
@@ -1875,7 +1878,7 @@
       <c r="G33" s="14"/>
     </row>
     <row r="34" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A34" s="47"/>
+      <c r="A34" s="43"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
@@ -1902,7 +1905,7 @@
       <c r="G35" s="14"/>
     </row>
     <row r="36" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A36" s="46" t="s">
+      <c r="A36" s="42" t="s">
         <v>9</v>
       </c>
       <c r="B36" s="5" t="s">
@@ -1921,7 +1924,7 @@
       <c r="G36" s="14"/>
     </row>
     <row r="37" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A37" s="47"/>
+      <c r="A37" s="43"/>
       <c r="B37" s="5" t="s">
         <v>22</v>
       </c>
@@ -1938,7 +1941,7 @@
       <c r="G37" s="14"/>
     </row>
     <row r="38" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A38" s="47"/>
+      <c r="A38" s="43"/>
       <c r="B38" s="5" t="s">
         <v>22</v>
       </c>
@@ -1957,7 +1960,7 @@
       <c r="G38" s="14"/>
     </row>
     <row r="39" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A39" s="47"/>
+      <c r="A39" s="43"/>
       <c r="B39" s="5" t="s">
         <v>22</v>
       </c>
@@ -1976,7 +1979,7 @@
       <c r="G39" s="14"/>
     </row>
     <row r="40" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A40" s="47"/>
+      <c r="A40" s="43"/>
       <c r="B40" s="5"/>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
@@ -2001,12 +2004,12 @@
       <c r="G41" s="14"/>
     </row>
     <row r="42" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="45" t="s">
+      <c r="A42" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="B42" s="48"/>
-      <c r="C42" s="48"/>
-      <c r="D42" s="49"/>
+      <c r="B42" s="44"/>
+      <c r="C42" s="44"/>
+      <c r="D42" s="45"/>
       <c r="E42" s="17"/>
       <c r="F42" s="17" t="s">
         <v>12</v>
@@ -2017,36 +2020,36 @@
       </c>
     </row>
     <row r="43" spans="1:7" s="10" customFormat="1" ht="82.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="40" t="s">
+      <c r="A43" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="B43" s="41"/>
-      <c r="C43" s="41"/>
-      <c r="D43" s="41"/>
-      <c r="E43" s="41"/>
-      <c r="F43" s="41"/>
-      <c r="G43" s="42"/>
+      <c r="B43" s="37"/>
+      <c r="C43" s="37"/>
+      <c r="D43" s="37"/>
+      <c r="E43" s="37"/>
+      <c r="F43" s="37"/>
+      <c r="G43" s="38"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="37"/>
-      <c r="B46" s="37"/>
-      <c r="C46" s="39"/>
-      <c r="D46" s="37"/>
-      <c r="E46" s="37"/>
+      <c r="A46" s="48"/>
+      <c r="B46" s="48"/>
+      <c r="C46" s="49"/>
+      <c r="D46" s="48"/>
+      <c r="E46" s="48"/>
       <c r="F46" s="23"/>
       <c r="G46" s="23"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="37"/>
-      <c r="B47" s="37"/>
-      <c r="C47" s="39"/>
-      <c r="D47" s="37"/>
-      <c r="E47" s="37"/>
+      <c r="A47" s="48"/>
+      <c r="B47" s="48"/>
+      <c r="C47" s="49"/>
+      <c r="D47" s="48"/>
+      <c r="E47" s="48"/>
       <c r="F47" s="23"/>
       <c r="G47" s="23"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="36"/>
+      <c r="A48" s="50"/>
       <c r="B48" s="25"/>
       <c r="C48" s="25"/>
       <c r="D48" s="25"/>
@@ -2055,7 +2058,7 @@
       <c r="G48" s="10"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="36"/>
+      <c r="A49" s="50"/>
       <c r="B49" s="25"/>
       <c r="C49" s="25"/>
       <c r="D49" s="25"/>
@@ -2064,7 +2067,7 @@
       <c r="G49" s="10"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="36"/>
+      <c r="A50" s="50"/>
       <c r="B50" s="25"/>
       <c r="C50" s="25"/>
       <c r="D50" s="25"/>
@@ -2073,7 +2076,7 @@
       <c r="G50" s="10"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="36"/>
+      <c r="A51" s="50"/>
       <c r="B51" s="25"/>
       <c r="C51" s="25"/>
       <c r="D51" s="25"/>
@@ -2082,7 +2085,7 @@
       <c r="G51" s="10"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="36"/>
+      <c r="A52" s="50"/>
       <c r="B52" s="25"/>
       <c r="C52" s="25"/>
       <c r="D52" s="25"/>
@@ -2091,7 +2094,7 @@
       <c r="G52" s="10"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="36"/>
+      <c r="A53" s="50"/>
       <c r="B53" s="25"/>
       <c r="C53" s="25"/>
       <c r="D53" s="25"/>
@@ -2109,7 +2112,7 @@
       <c r="G54" s="10"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="36"/>
+      <c r="A55" s="50"/>
       <c r="B55" s="25"/>
       <c r="C55" s="25"/>
       <c r="D55" s="25"/>
@@ -2118,7 +2121,7 @@
       <c r="G55" s="10"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="36"/>
+      <c r="A56" s="50"/>
       <c r="B56" s="25"/>
       <c r="C56" s="25"/>
       <c r="D56" s="25"/>
@@ -2127,7 +2130,7 @@
       <c r="G56" s="10"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="36"/>
+      <c r="A57" s="50"/>
       <c r="B57" s="25"/>
       <c r="C57" s="25"/>
       <c r="D57" s="25"/>
@@ -2136,7 +2139,7 @@
       <c r="G57" s="10"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="36"/>
+      <c r="A58" s="50"/>
       <c r="B58" s="25"/>
       <c r="C58" s="25"/>
       <c r="D58" s="25"/>
@@ -2154,7 +2157,7 @@
       <c r="G59" s="10"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="36"/>
+      <c r="A60" s="50"/>
       <c r="B60" s="25"/>
       <c r="C60" s="25"/>
       <c r="D60" s="25"/>
@@ -2163,7 +2166,7 @@
       <c r="G60" s="10"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="36"/>
+      <c r="A61" s="50"/>
       <c r="B61" s="25"/>
       <c r="C61" s="25"/>
       <c r="D61" s="25"/>
@@ -2172,7 +2175,7 @@
       <c r="G61" s="10"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="36"/>
+      <c r="A62" s="50"/>
       <c r="B62" s="25"/>
       <c r="C62" s="25"/>
       <c r="D62" s="25"/>
@@ -2181,7 +2184,7 @@
       <c r="G62" s="10"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="36"/>
+      <c r="A63" s="50"/>
       <c r="B63" s="25"/>
       <c r="C63" s="25"/>
       <c r="D63" s="25"/>
@@ -2199,7 +2202,7 @@
       <c r="G64" s="10"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" s="36"/>
+      <c r="A65" s="50"/>
       <c r="B65" s="25"/>
       <c r="C65" s="25"/>
       <c r="D65" s="25"/>
@@ -2208,7 +2211,7 @@
       <c r="G65" s="10"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" s="36"/>
+      <c r="A66" s="50"/>
       <c r="B66" s="25"/>
       <c r="C66" s="25"/>
       <c r="D66" s="25"/>
@@ -2217,7 +2220,7 @@
       <c r="G66" s="10"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" s="36"/>
+      <c r="A67" s="50"/>
       <c r="B67" s="25"/>
       <c r="C67" s="25"/>
       <c r="D67" s="25"/>
@@ -2226,7 +2229,7 @@
       <c r="G67" s="10"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" s="36"/>
+      <c r="A68" s="50"/>
       <c r="B68" s="25"/>
       <c r="C68" s="25"/>
       <c r="D68" s="25"/>
@@ -2244,7 +2247,7 @@
       <c r="G69" s="10"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" s="36"/>
+      <c r="A70" s="50"/>
       <c r="B70" s="25"/>
       <c r="C70" s="25"/>
       <c r="D70" s="25"/>
@@ -2253,7 +2256,7 @@
       <c r="G70" s="10"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" s="36"/>
+      <c r="A71" s="50"/>
       <c r="B71" s="25"/>
       <c r="C71" s="25"/>
       <c r="D71" s="25"/>
@@ -2262,7 +2265,7 @@
       <c r="G71" s="10"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" s="36"/>
+      <c r="A72" s="50"/>
       <c r="B72" s="25"/>
       <c r="C72" s="25"/>
       <c r="D72" s="25"/>
@@ -2271,7 +2274,7 @@
       <c r="G72" s="10"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A73" s="36"/>
+      <c r="A73" s="50"/>
       <c r="B73" s="25"/>
       <c r="C73" s="25"/>
       <c r="D73" s="25"/>
@@ -2289,25 +2292,37 @@
       <c r="G74" s="10"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" s="37"/>
-      <c r="B75" s="37"/>
-      <c r="C75" s="37"/>
-      <c r="D75" s="37"/>
+      <c r="A75" s="48"/>
+      <c r="B75" s="48"/>
+      <c r="C75" s="48"/>
+      <c r="D75" s="48"/>
       <c r="E75" s="27"/>
       <c r="F75" s="27"/>
       <c r="G75" s="28"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" s="38"/>
-      <c r="B76" s="38"/>
-      <c r="C76" s="38"/>
-      <c r="D76" s="38"/>
-      <c r="E76" s="38"/>
-      <c r="F76" s="38"/>
-      <c r="G76" s="38"/>
+      <c r="A76" s="51"/>
+      <c r="B76" s="51"/>
+      <c r="C76" s="51"/>
+      <c r="D76" s="51"/>
+      <c r="E76" s="51"/>
+      <c r="F76" s="51"/>
+      <c r="G76" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A48:A53"/>
+    <mergeCell ref="A75:D75"/>
+    <mergeCell ref="A76:G76"/>
+    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="A60:A63"/>
+    <mergeCell ref="A65:A68"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="E46:E47"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
@@ -2320,18 +2335,6 @@
     <mergeCell ref="A36:A40"/>
     <mergeCell ref="A42:D42"/>
     <mergeCell ref="A13:A19"/>
-    <mergeCell ref="A46:A47"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="E46:E47"/>
-    <mergeCell ref="A48:A53"/>
-    <mergeCell ref="A75:D75"/>
-    <mergeCell ref="A76:G76"/>
-    <mergeCell ref="A55:A58"/>
-    <mergeCell ref="A60:A63"/>
-    <mergeCell ref="A65:A68"/>
-    <mergeCell ref="A70:A73"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F16 F20:F41">
     <cfRule type="containsText" dxfId="31" priority="1" operator="containsText" text="Terminé">
@@ -2412,19 +2415,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="C3" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="43" t="s">
+      <c r="D3" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="45" t="s">
+      <c r="E3" s="41" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -2435,11 +2438,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="43"/>
-      <c r="B4" s="43"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="45"/>
+      <c r="A4" s="39"/>
+      <c r="B4" s="39"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -2448,7 +2451,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="42" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -2467,7 +2470,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A6" s="47"/>
+      <c r="A6" s="43"/>
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
@@ -2484,7 +2487,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" s="10" customFormat="1" ht="90" x14ac:dyDescent="0.2">
-      <c r="A7" s="47"/>
+      <c r="A7" s="43"/>
       <c r="B7" s="5" t="s">
         <v>22</v>
       </c>
@@ -2503,7 +2506,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="47"/>
+      <c r="A8" s="43"/>
       <c r="B8" s="5" t="s">
         <v>22</v>
       </c>
@@ -2520,7 +2523,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="47"/>
+      <c r="A9" s="43"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -2529,7 +2532,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="47"/>
+      <c r="A10" s="43"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -2554,7 +2557,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A12" s="47" t="s">
+      <c r="A12" s="43" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="5" t="s">
@@ -2573,7 +2576,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" s="10" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
-      <c r="A13" s="47"/>
+      <c r="A13" s="43"/>
       <c r="B13" s="5" t="s">
         <v>22</v>
       </c>
@@ -2590,7 +2593,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A14" s="47"/>
+      <c r="A14" s="43"/>
       <c r="B14" s="5" t="s">
         <v>22</v>
       </c>
@@ -2607,7 +2610,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A15" s="47"/>
+      <c r="A15" s="43"/>
       <c r="B15" s="5" t="s">
         <v>22</v>
       </c>
@@ -2624,7 +2627,7 @@
       <c r="G15" s="14"/>
     </row>
     <row r="16" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="47"/>
+      <c r="A16" s="43"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
@@ -2649,7 +2652,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:10" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A18" s="47" t="s">
+      <c r="A18" s="43" t="s">
         <v>7</v>
       </c>
       <c r="B18" s="5" t="s">
@@ -2669,7 +2672,7 @@
       <c r="J18" s="32"/>
     </row>
     <row r="19" spans="1:10" s="10" customFormat="1" ht="146.25" x14ac:dyDescent="0.2">
-      <c r="A19" s="47"/>
+      <c r="A19" s="43"/>
       <c r="B19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2686,7 +2689,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:10" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A20" s="47"/>
+      <c r="A20" s="43"/>
       <c r="B20" s="5" t="s">
         <v>22</v>
       </c>
@@ -2703,7 +2706,7 @@
       <c r="G20" s="14"/>
     </row>
     <row r="21" spans="1:10" s="10" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="47"/>
+      <c r="A21" s="43"/>
       <c r="B21" s="5" t="s">
         <v>22</v>
       </c>
@@ -2711,7 +2714,7 @@
         <v>26</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="6">
@@ -2720,7 +2723,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:10" s="10" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="47"/>
+      <c r="A22" s="43"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
@@ -2745,28 +2748,44 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:10" s="10" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="47" t="s">
+      <c r="A24" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
+      <c r="B24" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="E24" s="4"/>
-      <c r="F24" s="6"/>
+      <c r="F24" s="13">
+        <v>0.2</v>
+      </c>
       <c r="G24" s="14"/>
     </row>
-    <row r="25" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A25" s="47"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
+    <row r="25" spans="1:10" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
+      <c r="A25" s="43"/>
+      <c r="B25" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>73</v>
+      </c>
       <c r="E25" s="4"/>
-      <c r="F25" s="6"/>
+      <c r="F25" s="6">
+        <v>1.3</v>
+      </c>
       <c r="G25" s="14"/>
       <c r="J25" s="32"/>
     </row>
     <row r="26" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="47"/>
+      <c r="A26" s="43"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
@@ -2776,7 +2795,7 @@
       <c r="J26" s="32"/>
     </row>
     <row r="27" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="47"/>
+      <c r="A27" s="43"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
       <c r="D27" s="4"/>
@@ -2796,12 +2815,12 @@
       </c>
       <c r="F28" s="18">
         <f>SUM(F24:F27)</f>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A29" s="47" t="s">
+      <c r="A29" s="43" t="s">
         <v>9</v>
       </c>
       <c r="B29" s="4"/>
@@ -2812,7 +2831,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A30" s="47"/>
+      <c r="A30" s="43"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -2821,7 +2840,7 @@
       <c r="G30" s="14"/>
     </row>
     <row r="31" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A31" s="47"/>
+      <c r="A31" s="43"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
@@ -2830,7 +2849,7 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="47"/>
+      <c r="A32" s="43"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
@@ -2855,31 +2874,31 @@
       <c r="G33" s="14"/>
     </row>
     <row r="34" spans="1:7" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="43" t="s">
+      <c r="A34" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="B34" s="43"/>
-      <c r="C34" s="43"/>
-      <c r="D34" s="43"/>
+      <c r="B34" s="39"/>
+      <c r="C34" s="39"/>
+      <c r="D34" s="39"/>
       <c r="E34" s="17"/>
       <c r="F34" s="17" t="s">
         <v>12</v>
       </c>
       <c r="G34" s="22">
         <f>F11+F17+F23+F28+F33</f>
-        <v>21</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="40" t="s">
+      <c r="A35" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="B35" s="41"/>
-      <c r="C35" s="41"/>
-      <c r="D35" s="41"/>
-      <c r="E35" s="41"/>
-      <c r="F35" s="41"/>
-      <c r="G35" s="42"/>
+      <c r="B35" s="37"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="37"/>
+      <c r="F35" s="37"/>
+      <c r="G35" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -2954,19 +2973,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="C3" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="43" t="s">
+      <c r="D3" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="45" t="s">
+      <c r="E3" s="41" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -2977,11 +2996,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="43"/>
-      <c r="B4" s="43"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="45"/>
+      <c r="A4" s="39"/>
+      <c r="B4" s="39"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -2990,7 +3009,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="42" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -3001,7 +3020,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="47"/>
+      <c r="A6" s="43"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -3010,7 +3029,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="47"/>
+      <c r="A7" s="43"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -3019,7 +3038,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="47"/>
+      <c r="A8" s="43"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -3028,7 +3047,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="47"/>
+      <c r="A9" s="43"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="E9" s="4"/>
@@ -3036,7 +3055,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="47"/>
+      <c r="A10" s="43"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -3061,7 +3080,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="47" t="s">
+      <c r="A12" s="43" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -3072,7 +3091,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="47"/>
+      <c r="A13" s="43"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -3081,7 +3100,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="47"/>
+      <c r="A14" s="43"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -3090,7 +3109,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="47"/>
+      <c r="A15" s="43"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -3115,7 +3134,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="47" t="s">
+      <c r="A17" s="43" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -3126,7 +3145,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="47"/>
+      <c r="A18" s="43"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -3135,7 +3154,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="47"/>
+      <c r="A19" s="43"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -3144,7 +3163,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="47"/>
+      <c r="A20" s="43"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -3169,7 +3188,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="47" t="s">
+      <c r="A22" s="43" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -3180,7 +3199,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="47"/>
+      <c r="A23" s="43"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -3189,7 +3208,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="47"/>
+      <c r="A24" s="43"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -3198,7 +3217,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="47"/>
+      <c r="A25" s="43"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -3223,7 +3242,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="47" t="s">
+      <c r="A27" s="43" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -3234,7 +3253,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="47"/>
+      <c r="A28" s="43"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -3243,7 +3262,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="47"/>
+      <c r="A29" s="43"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -3252,7 +3271,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="47"/>
+      <c r="A30" s="43"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -3277,12 +3296,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="43" t="s">
+      <c r="A32" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="43"/>
-      <c r="C32" s="43"/>
-      <c r="D32" s="43"/>
+      <c r="B32" s="39"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="39"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -3293,18 +3312,23 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="40" t="s">
+      <c r="A33" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="41"/>
-      <c r="C33" s="41"/>
-      <c r="D33" s="41"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="42"/>
+      <c r="B33" s="37"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A5:A10"/>
@@ -3312,11 +3336,6 @@
     <mergeCell ref="A17:A20"/>
     <mergeCell ref="A22:A25"/>
     <mergeCell ref="A27:A30"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F31">
     <cfRule type="containsText" dxfId="19" priority="1" operator="containsText" text="Terminé">
@@ -3374,19 +3393,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="C3" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="43" t="s">
+      <c r="D3" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="45" t="s">
+      <c r="E3" s="41" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -3397,11 +3416,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="43"/>
-      <c r="B4" s="43"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="45"/>
+      <c r="A4" s="39"/>
+      <c r="B4" s="39"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -3410,7 +3429,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="42" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -3421,7 +3440,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="47"/>
+      <c r="A6" s="43"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -3430,7 +3449,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="47"/>
+      <c r="A7" s="43"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -3439,7 +3458,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="47"/>
+      <c r="A8" s="43"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -3448,7 +3467,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="47"/>
+      <c r="A9" s="43"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -3457,7 +3476,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="47"/>
+      <c r="A10" s="43"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -3482,7 +3501,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="47" t="s">
+      <c r="A12" s="43" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -3493,7 +3512,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="47"/>
+      <c r="A13" s="43"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -3502,7 +3521,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="47"/>
+      <c r="A14" s="43"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -3511,7 +3530,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="47"/>
+      <c r="A15" s="43"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -3536,7 +3555,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="47" t="s">
+      <c r="A17" s="43" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -3547,7 +3566,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="47"/>
+      <c r="A18" s="43"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -3556,7 +3575,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="47"/>
+      <c r="A19" s="43"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -3565,7 +3584,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="47"/>
+      <c r="A20" s="43"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -3590,7 +3609,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="47" t="s">
+      <c r="A22" s="43" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -3601,7 +3620,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="47"/>
+      <c r="A23" s="43"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -3610,7 +3629,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="47"/>
+      <c r="A24" s="43"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -3619,7 +3638,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="47"/>
+      <c r="A25" s="43"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -3644,7 +3663,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="47" t="s">
+      <c r="A27" s="43" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -3655,7 +3674,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="47"/>
+      <c r="A28" s="43"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -3664,7 +3683,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="47"/>
+      <c r="A29" s="43"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -3673,7 +3692,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="47"/>
+      <c r="A30" s="43"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -3698,12 +3717,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="43" t="s">
+      <c r="A32" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="43"/>
-      <c r="C32" s="43"/>
-      <c r="D32" s="43"/>
+      <c r="B32" s="39"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="39"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -3714,18 +3733,23 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="40" t="s">
+      <c r="A33" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="41"/>
-      <c r="C33" s="41"/>
-      <c r="D33" s="41"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="42"/>
+      <c r="B33" s="37"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A5:A10"/>
@@ -3733,11 +3757,6 @@
     <mergeCell ref="A17:A20"/>
     <mergeCell ref="A22:A25"/>
     <mergeCell ref="A27:A30"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F31">
     <cfRule type="containsText" dxfId="15" priority="1" operator="containsText" text="Terminé">
@@ -3795,19 +3814,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="C3" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="43" t="s">
+      <c r="D3" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="45" t="s">
+      <c r="E3" s="41" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -3818,11 +3837,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="43"/>
-      <c r="B4" s="43"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="45"/>
+      <c r="A4" s="39"/>
+      <c r="B4" s="39"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -3831,7 +3850,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="42" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -3842,7 +3861,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="47"/>
+      <c r="A6" s="43"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -3851,7 +3870,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="47"/>
+      <c r="A7" s="43"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -3860,7 +3879,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="47"/>
+      <c r="A8" s="43"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -3869,7 +3888,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="47"/>
+      <c r="A9" s="43"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -3878,7 +3897,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="47"/>
+      <c r="A10" s="43"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -3903,7 +3922,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="47" t="s">
+      <c r="A12" s="43" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -3914,7 +3933,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="47"/>
+      <c r="A13" s="43"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -3923,7 +3942,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="47"/>
+      <c r="A14" s="43"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -3932,7 +3951,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="47"/>
+      <c r="A15" s="43"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -3957,7 +3976,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="47" t="s">
+      <c r="A17" s="43" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -3968,7 +3987,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="47"/>
+      <c r="A18" s="43"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -3977,7 +3996,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="47"/>
+      <c r="A19" s="43"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -3986,7 +4005,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="47"/>
+      <c r="A20" s="43"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -4011,7 +4030,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="47" t="s">
+      <c r="A22" s="43" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -4022,7 +4041,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="47"/>
+      <c r="A23" s="43"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -4031,7 +4050,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="47"/>
+      <c r="A24" s="43"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -4040,7 +4059,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="47"/>
+      <c r="A25" s="43"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -4065,7 +4084,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="47" t="s">
+      <c r="A27" s="43" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -4076,7 +4095,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="47"/>
+      <c r="A28" s="43"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -4085,7 +4104,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="47"/>
+      <c r="A29" s="43"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -4094,7 +4113,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="47"/>
+      <c r="A30" s="43"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -4119,12 +4138,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="43" t="s">
+      <c r="A32" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="43"/>
-      <c r="C32" s="43"/>
-      <c r="D32" s="43"/>
+      <c r="B32" s="39"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="39"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -4135,15 +4154,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="40" t="s">
+      <c r="A33" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="41"/>
-      <c r="C33" s="41"/>
-      <c r="D33" s="41"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="42"/>
+      <c r="B33" s="37"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -4218,19 +4237,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="C3" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="43" t="s">
+      <c r="D3" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="45" t="s">
+      <c r="E3" s="41" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -4241,11 +4260,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="43"/>
-      <c r="B4" s="43"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="45"/>
+      <c r="A4" s="39"/>
+      <c r="B4" s="39"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -4254,7 +4273,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="42" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -4265,7 +4284,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="47"/>
+      <c r="A6" s="43"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -4274,7 +4293,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="47"/>
+      <c r="A7" s="43"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -4283,7 +4302,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="47"/>
+      <c r="A8" s="43"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -4292,7 +4311,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="47"/>
+      <c r="A9" s="43"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -4301,7 +4320,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="47"/>
+      <c r="A10" s="43"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -4326,7 +4345,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="47" t="s">
+      <c r="A12" s="43" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -4337,7 +4356,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="47"/>
+      <c r="A13" s="43"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -4346,7 +4365,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="47"/>
+      <c r="A14" s="43"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -4355,7 +4374,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="47"/>
+      <c r="A15" s="43"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -4380,7 +4399,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="47" t="s">
+      <c r="A17" s="43" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -4391,7 +4410,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="47"/>
+      <c r="A18" s="43"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -4400,7 +4419,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="47"/>
+      <c r="A19" s="43"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -4409,7 +4428,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="47"/>
+      <c r="A20" s="43"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -4434,7 +4453,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="47" t="s">
+      <c r="A22" s="43" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -4445,7 +4464,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="47"/>
+      <c r="A23" s="43"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -4454,7 +4473,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="47"/>
+      <c r="A24" s="43"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -4463,7 +4482,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="47"/>
+      <c r="A25" s="43"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -4488,7 +4507,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="47" t="s">
+      <c r="A27" s="43" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -4499,7 +4518,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="47"/>
+      <c r="A28" s="43"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -4508,7 +4527,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="47"/>
+      <c r="A29" s="43"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -4517,7 +4536,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="47"/>
+      <c r="A30" s="43"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -4542,12 +4561,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="43" t="s">
+      <c r="A32" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="43"/>
-      <c r="C32" s="43"/>
-      <c r="D32" s="43"/>
+      <c r="B32" s="39"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="39"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -4558,15 +4577,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="40" t="s">
+      <c r="A33" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="41"/>
-      <c r="C33" s="41"/>
-      <c r="D33" s="41"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="42"/>
+      <c r="B33" s="37"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -4639,19 +4658,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="C3" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="43" t="s">
+      <c r="D3" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="45" t="s">
+      <c r="E3" s="41" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -4662,11 +4681,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="43"/>
-      <c r="B4" s="43"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="45"/>
+      <c r="A4" s="39"/>
+      <c r="B4" s="39"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -4675,7 +4694,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="42" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -4686,7 +4705,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="47"/>
+      <c r="A6" s="43"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -4695,7 +4714,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="47"/>
+      <c r="A7" s="43"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="E7" s="5"/>
@@ -4703,7 +4722,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="47"/>
+      <c r="A8" s="43"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -4712,7 +4731,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="47"/>
+      <c r="A9" s="43"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -4721,7 +4740,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="47"/>
+      <c r="A10" s="43"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -4746,7 +4765,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="47" t="s">
+      <c r="A12" s="43" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -4757,7 +4776,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="47"/>
+      <c r="A13" s="43"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -4766,7 +4785,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="47"/>
+      <c r="A14" s="43"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -4775,7 +4794,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="47"/>
+      <c r="A15" s="43"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -4800,7 +4819,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="47" t="s">
+      <c r="A17" s="43" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -4811,7 +4830,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="47"/>
+      <c r="A18" s="43"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -4820,7 +4839,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="47"/>
+      <c r="A19" s="43"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -4829,7 +4848,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="47"/>
+      <c r="A20" s="43"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -4854,7 +4873,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="47" t="s">
+      <c r="A22" s="43" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -4865,7 +4884,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="47"/>
+      <c r="A23" s="43"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -4874,7 +4893,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="47"/>
+      <c r="A24" s="43"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -4883,7 +4902,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="47"/>
+      <c r="A25" s="43"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -4908,7 +4927,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="47" t="s">
+      <c r="A27" s="43" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -4919,7 +4938,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="47"/>
+      <c r="A28" s="43"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -4928,7 +4947,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="47"/>
+      <c r="A29" s="43"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -4937,7 +4956,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="47"/>
+      <c r="A30" s="43"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -4962,12 +4981,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="43" t="s">
+      <c r="A32" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="43"/>
-      <c r="C32" s="43"/>
-      <c r="D32" s="43"/>
+      <c r="B32" s="39"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="39"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -4978,15 +4997,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="40" t="s">
+      <c r="A33" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="41"/>
-      <c r="C33" s="41"/>
-      <c r="D33" s="41"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="42"/>
+      <c r="B33" s="37"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
début de la programmation sur le STM32
tests pour apprendre le fonctionnement de l'IDE de STM32
</commit_message>
<xml_diff>
--- a/jeu_du_moulin_boura/rpt/jeu-du-moulin-bourquenouda-rpt-journal.xlsx
+++ b/jeu_du_moulin_boura/rpt/jeu-du-moulin-bourquenouda-rpt-journal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/alexandre_bourquenoud_studentfr_ch/Documents/PHIE/jeu_du_moulin_alexandre_bourquenoud/jeu_du_moulin_2025_boura/jeu_du_moulin_boura/rpt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="154" documentId="13_ncr:1_{ED970C68-2653-443C-99A4-F9D694477206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D33F6F5-A8DD-402B-9B04-39EFC4D80797}"/>
+  <xr:revisionPtr revIDLastSave="171" documentId="13_ncr:1_{ED970C68-2653-443C-99A4-F9D694477206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6784FB9-F2DE-435C-B4E3-6D0B34FC41D9}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="s1" sheetId="8" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="80">
   <si>
     <t>Date</t>
   </si>
@@ -334,6 +334,21 @@
   </si>
   <si>
     <t>finission des dernier détails du pcb par example amélioration du routage des pistes et création des Gerber et vérification sur eurocircuit de la classe et validité du circuit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revue du programme crée par M.Egli et du mon ancien code pour matrice de LEDs pour voir si c'est possible de l'implementer sur le STM32 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise au point de la progression du projet avec M.Cunha et  ensuite </t>
+  </si>
+  <si>
+    <t>Problème de connexion qui m'empèche de debugger sur la plaque fourni par M.Egli</t>
+  </si>
+  <si>
+    <t>programmation des touches et LED pour que ce soir conforme a ce qu'on me demande dans le cahier des charges</t>
+  </si>
+  <si>
+    <t>essaie debugger le programme de test de M.Egli pour comprendre le fonctionnement de STM32CubeIDE</t>
   </si>
 </sst>
 </file>
@@ -620,6 +635,18 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -655,18 +682,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1350,19 +1365,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="45" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -1373,11 +1388,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="41"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -1386,7 +1401,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" s="10" customFormat="1" ht="78.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="46" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -1407,7 +1422,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A6" s="43"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
@@ -1424,7 +1439,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="43"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="5" t="s">
         <v>22</v>
       </c>
@@ -1441,7 +1456,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="43"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="5" t="s">
         <v>22</v>
       </c>
@@ -1458,7 +1473,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A9" s="43"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="5" t="s">
         <v>22</v>
       </c>
@@ -1475,7 +1490,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" s="10" customFormat="1" ht="78.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="43"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="5" t="s">
         <v>22</v>
       </c>
@@ -1494,7 +1509,7 @@
       <c r="G10" s="14"/>
     </row>
     <row r="11" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A11" s="43"/>
+      <c r="A11" s="47"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -1519,7 +1534,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A13" s="46" t="s">
+      <c r="A13" s="50" t="s">
         <v>5</v>
       </c>
       <c r="B13" s="5" t="s">
@@ -1538,7 +1553,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A14" s="47"/>
+      <c r="A14" s="51"/>
       <c r="B14" s="5" t="s">
         <v>22</v>
       </c>
@@ -1555,7 +1570,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="47"/>
+      <c r="A15" s="51"/>
       <c r="B15" s="5" t="s">
         <v>22</v>
       </c>
@@ -1572,7 +1587,7 @@
       <c r="G15" s="14"/>
     </row>
     <row r="16" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A16" s="47"/>
+      <c r="A16" s="51"/>
       <c r="B16" s="5" t="s">
         <v>22</v>
       </c>
@@ -1589,7 +1604,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A17" s="47"/>
+      <c r="A17" s="51"/>
       <c r="B17" s="5" t="s">
         <v>22</v>
       </c>
@@ -1606,7 +1621,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="47"/>
+      <c r="A18" s="51"/>
       <c r="B18" s="5" t="s">
         <v>22</v>
       </c>
@@ -1623,7 +1638,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A19" s="47"/>
+      <c r="A19" s="51"/>
       <c r="B19" s="5"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -1648,7 +1663,7 @@
       <c r="G20" s="14"/>
     </row>
     <row r="21" spans="1:7" s="10" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
-      <c r="A21" s="42" t="s">
+      <c r="A21" s="46" t="s">
         <v>7</v>
       </c>
       <c r="B21" s="5" t="s">
@@ -1667,7 +1682,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="43"/>
+      <c r="A22" s="47"/>
       <c r="B22" s="5" t="s">
         <v>22</v>
       </c>
@@ -1684,7 +1699,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A23" s="43"/>
+      <c r="A23" s="47"/>
       <c r="B23" s="5" t="s">
         <v>22</v>
       </c>
@@ -1701,7 +1716,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A24" s="43"/>
+      <c r="A24" s="47"/>
       <c r="B24" s="5" t="s">
         <v>22</v>
       </c>
@@ -1718,7 +1733,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A25" s="43"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="5" t="s">
         <v>22</v>
       </c>
@@ -1735,7 +1750,7 @@
       <c r="G25" s="14"/>
     </row>
     <row r="26" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="43"/>
+      <c r="A26" s="47"/>
       <c r="B26" s="5" t="s">
         <v>22</v>
       </c>
@@ -1754,7 +1769,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A27" s="43"/>
+      <c r="A27" s="47"/>
       <c r="B27" s="5" t="s">
         <v>22</v>
       </c>
@@ -1787,7 +1802,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A29" s="42" t="s">
+      <c r="A29" s="46" t="s">
         <v>8</v>
       </c>
       <c r="B29" s="5" t="s">
@@ -1806,7 +1821,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A30" s="43"/>
+      <c r="A30" s="47"/>
       <c r="B30" s="5" t="s">
         <v>22</v>
       </c>
@@ -1825,7 +1840,7 @@
       <c r="G30" s="14"/>
     </row>
     <row r="31" spans="1:7" s="10" customFormat="1" ht="90" x14ac:dyDescent="0.2">
-      <c r="A31" s="43"/>
+      <c r="A31" s="47"/>
       <c r="B31" s="5" t="s">
         <v>22</v>
       </c>
@@ -1844,7 +1859,7 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" s="10" customFormat="1" ht="78.75" x14ac:dyDescent="0.2">
-      <c r="A32" s="43"/>
+      <c r="A32" s="47"/>
       <c r="B32" s="5" t="s">
         <v>22</v>
       </c>
@@ -1861,7 +1876,7 @@
       <c r="G32" s="14"/>
     </row>
     <row r="33" spans="1:7" s="10" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
-      <c r="A33" s="43"/>
+      <c r="A33" s="47"/>
       <c r="B33" s="5" t="s">
         <v>22</v>
       </c>
@@ -1878,7 +1893,7 @@
       <c r="G33" s="14"/>
     </row>
     <row r="34" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A34" s="43"/>
+      <c r="A34" s="47"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
@@ -1905,7 +1920,7 @@
       <c r="G35" s="14"/>
     </row>
     <row r="36" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A36" s="42" t="s">
+      <c r="A36" s="46" t="s">
         <v>9</v>
       </c>
       <c r="B36" s="5" t="s">
@@ -1924,7 +1939,7 @@
       <c r="G36" s="14"/>
     </row>
     <row r="37" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A37" s="43"/>
+      <c r="A37" s="47"/>
       <c r="B37" s="5" t="s">
         <v>22</v>
       </c>
@@ -1941,7 +1956,7 @@
       <c r="G37" s="14"/>
     </row>
     <row r="38" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A38" s="43"/>
+      <c r="A38" s="47"/>
       <c r="B38" s="5" t="s">
         <v>22</v>
       </c>
@@ -1960,7 +1975,7 @@
       <c r="G38" s="14"/>
     </row>
     <row r="39" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A39" s="43"/>
+      <c r="A39" s="47"/>
       <c r="B39" s="5" t="s">
         <v>22</v>
       </c>
@@ -1979,7 +1994,7 @@
       <c r="G39" s="14"/>
     </row>
     <row r="40" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A40" s="43"/>
+      <c r="A40" s="47"/>
       <c r="B40" s="5"/>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
@@ -2004,12 +2019,12 @@
       <c r="G41" s="14"/>
     </row>
     <row r="42" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="41" t="s">
+      <c r="A42" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="B42" s="44"/>
-      <c r="C42" s="44"/>
-      <c r="D42" s="45"/>
+      <c r="B42" s="48"/>
+      <c r="C42" s="48"/>
+      <c r="D42" s="49"/>
       <c r="E42" s="17"/>
       <c r="F42" s="17" t="s">
         <v>12</v>
@@ -2020,36 +2035,36 @@
       </c>
     </row>
     <row r="43" spans="1:7" s="10" customFormat="1" ht="82.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="36" t="s">
+      <c r="A43" s="40" t="s">
         <v>62</v>
       </c>
-      <c r="B43" s="37"/>
-      <c r="C43" s="37"/>
-      <c r="D43" s="37"/>
-      <c r="E43" s="37"/>
-      <c r="F43" s="37"/>
-      <c r="G43" s="38"/>
+      <c r="B43" s="41"/>
+      <c r="C43" s="41"/>
+      <c r="D43" s="41"/>
+      <c r="E43" s="41"/>
+      <c r="F43" s="41"/>
+      <c r="G43" s="42"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="48"/>
-      <c r="B46" s="48"/>
-      <c r="C46" s="49"/>
-      <c r="D46" s="48"/>
-      <c r="E46" s="48"/>
+      <c r="A46" s="37"/>
+      <c r="B46" s="37"/>
+      <c r="C46" s="39"/>
+      <c r="D46" s="37"/>
+      <c r="E46" s="37"/>
       <c r="F46" s="23"/>
       <c r="G46" s="23"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="48"/>
-      <c r="B47" s="48"/>
-      <c r="C47" s="49"/>
-      <c r="D47" s="48"/>
-      <c r="E47" s="48"/>
+      <c r="A47" s="37"/>
+      <c r="B47" s="37"/>
+      <c r="C47" s="39"/>
+      <c r="D47" s="37"/>
+      <c r="E47" s="37"/>
       <c r="F47" s="23"/>
       <c r="G47" s="23"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="50"/>
+      <c r="A48" s="36"/>
       <c r="B48" s="25"/>
       <c r="C48" s="25"/>
       <c r="D48" s="25"/>
@@ -2058,7 +2073,7 @@
       <c r="G48" s="10"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="50"/>
+      <c r="A49" s="36"/>
       <c r="B49" s="25"/>
       <c r="C49" s="25"/>
       <c r="D49" s="25"/>
@@ -2067,7 +2082,7 @@
       <c r="G49" s="10"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="50"/>
+      <c r="A50" s="36"/>
       <c r="B50" s="25"/>
       <c r="C50" s="25"/>
       <c r="D50" s="25"/>
@@ -2076,7 +2091,7 @@
       <c r="G50" s="10"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="50"/>
+      <c r="A51" s="36"/>
       <c r="B51" s="25"/>
       <c r="C51" s="25"/>
       <c r="D51" s="25"/>
@@ -2085,7 +2100,7 @@
       <c r="G51" s="10"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="50"/>
+      <c r="A52" s="36"/>
       <c r="B52" s="25"/>
       <c r="C52" s="25"/>
       <c r="D52" s="25"/>
@@ -2094,7 +2109,7 @@
       <c r="G52" s="10"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="50"/>
+      <c r="A53" s="36"/>
       <c r="B53" s="25"/>
       <c r="C53" s="25"/>
       <c r="D53" s="25"/>
@@ -2112,7 +2127,7 @@
       <c r="G54" s="10"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="50"/>
+      <c r="A55" s="36"/>
       <c r="B55" s="25"/>
       <c r="C55" s="25"/>
       <c r="D55" s="25"/>
@@ -2121,7 +2136,7 @@
       <c r="G55" s="10"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="50"/>
+      <c r="A56" s="36"/>
       <c r="B56" s="25"/>
       <c r="C56" s="25"/>
       <c r="D56" s="25"/>
@@ -2130,7 +2145,7 @@
       <c r="G56" s="10"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="50"/>
+      <c r="A57" s="36"/>
       <c r="B57" s="25"/>
       <c r="C57" s="25"/>
       <c r="D57" s="25"/>
@@ -2139,7 +2154,7 @@
       <c r="G57" s="10"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="50"/>
+      <c r="A58" s="36"/>
       <c r="B58" s="25"/>
       <c r="C58" s="25"/>
       <c r="D58" s="25"/>
@@ -2157,7 +2172,7 @@
       <c r="G59" s="10"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="50"/>
+      <c r="A60" s="36"/>
       <c r="B60" s="25"/>
       <c r="C60" s="25"/>
       <c r="D60" s="25"/>
@@ -2166,7 +2181,7 @@
       <c r="G60" s="10"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="50"/>
+      <c r="A61" s="36"/>
       <c r="B61" s="25"/>
       <c r="C61" s="25"/>
       <c r="D61" s="25"/>
@@ -2175,7 +2190,7 @@
       <c r="G61" s="10"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="50"/>
+      <c r="A62" s="36"/>
       <c r="B62" s="25"/>
       <c r="C62" s="25"/>
       <c r="D62" s="25"/>
@@ -2184,7 +2199,7 @@
       <c r="G62" s="10"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="50"/>
+      <c r="A63" s="36"/>
       <c r="B63" s="25"/>
       <c r="C63" s="25"/>
       <c r="D63" s="25"/>
@@ -2202,7 +2217,7 @@
       <c r="G64" s="10"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" s="50"/>
+      <c r="A65" s="36"/>
       <c r="B65" s="25"/>
       <c r="C65" s="25"/>
       <c r="D65" s="25"/>
@@ -2211,7 +2226,7 @@
       <c r="G65" s="10"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" s="50"/>
+      <c r="A66" s="36"/>
       <c r="B66" s="25"/>
       <c r="C66" s="25"/>
       <c r="D66" s="25"/>
@@ -2220,7 +2235,7 @@
       <c r="G66" s="10"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" s="50"/>
+      <c r="A67" s="36"/>
       <c r="B67" s="25"/>
       <c r="C67" s="25"/>
       <c r="D67" s="25"/>
@@ -2229,7 +2244,7 @@
       <c r="G67" s="10"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" s="50"/>
+      <c r="A68" s="36"/>
       <c r="B68" s="25"/>
       <c r="C68" s="25"/>
       <c r="D68" s="25"/>
@@ -2247,7 +2262,7 @@
       <c r="G69" s="10"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" s="50"/>
+      <c r="A70" s="36"/>
       <c r="B70" s="25"/>
       <c r="C70" s="25"/>
       <c r="D70" s="25"/>
@@ -2256,7 +2271,7 @@
       <c r="G70" s="10"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" s="50"/>
+      <c r="A71" s="36"/>
       <c r="B71" s="25"/>
       <c r="C71" s="25"/>
       <c r="D71" s="25"/>
@@ -2265,7 +2280,7 @@
       <c r="G71" s="10"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" s="50"/>
+      <c r="A72" s="36"/>
       <c r="B72" s="25"/>
       <c r="C72" s="25"/>
       <c r="D72" s="25"/>
@@ -2274,7 +2289,7 @@
       <c r="G72" s="10"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A73" s="50"/>
+      <c r="A73" s="36"/>
       <c r="B73" s="25"/>
       <c r="C73" s="25"/>
       <c r="D73" s="25"/>
@@ -2292,37 +2307,25 @@
       <c r="G74" s="10"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" s="48"/>
-      <c r="B75" s="48"/>
-      <c r="C75" s="48"/>
-      <c r="D75" s="48"/>
+      <c r="A75" s="37"/>
+      <c r="B75" s="37"/>
+      <c r="C75" s="37"/>
+      <c r="D75" s="37"/>
       <c r="E75" s="27"/>
       <c r="F75" s="27"/>
       <c r="G75" s="28"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" s="51"/>
-      <c r="B76" s="51"/>
-      <c r="C76" s="51"/>
-      <c r="D76" s="51"/>
-      <c r="E76" s="51"/>
-      <c r="F76" s="51"/>
-      <c r="G76" s="51"/>
+      <c r="A76" s="38"/>
+      <c r="B76" s="38"/>
+      <c r="C76" s="38"/>
+      <c r="D76" s="38"/>
+      <c r="E76" s="38"/>
+      <c r="F76" s="38"/>
+      <c r="G76" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A48:A53"/>
-    <mergeCell ref="A75:D75"/>
-    <mergeCell ref="A76:G76"/>
-    <mergeCell ref="A55:A58"/>
-    <mergeCell ref="A60:A63"/>
-    <mergeCell ref="A65:A68"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A46:A47"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="E46:E47"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
@@ -2335,6 +2338,18 @@
     <mergeCell ref="A36:A40"/>
     <mergeCell ref="A42:D42"/>
     <mergeCell ref="A13:A19"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="E46:E47"/>
+    <mergeCell ref="A48:A53"/>
+    <mergeCell ref="A75:D75"/>
+    <mergeCell ref="A76:G76"/>
+    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="A60:A63"/>
+    <mergeCell ref="A65:A68"/>
+    <mergeCell ref="A70:A73"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F16 F20:F41">
     <cfRule type="containsText" dxfId="31" priority="1" operator="containsText" text="Terminé">
@@ -2375,7 +2390,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" style="1" customWidth="1"/>
@@ -2415,19 +2430,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="45" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -2438,11 +2453,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="41"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -2451,7 +2466,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="46" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -2470,7 +2485,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A6" s="43"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
@@ -2487,7 +2502,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" s="10" customFormat="1" ht="90" x14ac:dyDescent="0.2">
-      <c r="A7" s="43"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="5" t="s">
         <v>22</v>
       </c>
@@ -2506,7 +2521,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="43"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="5" t="s">
         <v>22</v>
       </c>
@@ -2523,7 +2538,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="43"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -2532,7 +2547,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="43"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -2557,7 +2572,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="47" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="5" t="s">
@@ -2576,7 +2591,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" s="10" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
-      <c r="A13" s="43"/>
+      <c r="A13" s="47"/>
       <c r="B13" s="5" t="s">
         <v>22</v>
       </c>
@@ -2593,7 +2608,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A14" s="43"/>
+      <c r="A14" s="47"/>
       <c r="B14" s="5" t="s">
         <v>22</v>
       </c>
@@ -2610,7 +2625,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A15" s="43"/>
+      <c r="A15" s="47"/>
       <c r="B15" s="5" t="s">
         <v>22</v>
       </c>
@@ -2627,7 +2642,7 @@
       <c r="G15" s="14"/>
     </row>
     <row r="16" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="43"/>
+      <c r="A16" s="47"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
@@ -2652,7 +2667,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:10" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A18" s="43" t="s">
+      <c r="A18" s="47" t="s">
         <v>7</v>
       </c>
       <c r="B18" s="5" t="s">
@@ -2672,7 +2687,7 @@
       <c r="J18" s="32"/>
     </row>
     <row r="19" spans="1:10" s="10" customFormat="1" ht="146.25" x14ac:dyDescent="0.2">
-      <c r="A19" s="43"/>
+      <c r="A19" s="47"/>
       <c r="B19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2689,7 +2704,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:10" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A20" s="43"/>
+      <c r="A20" s="47"/>
       <c r="B20" s="5" t="s">
         <v>22</v>
       </c>
@@ -2706,7 +2721,7 @@
       <c r="G20" s="14"/>
     </row>
     <row r="21" spans="1:10" s="10" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="43"/>
+      <c r="A21" s="47"/>
       <c r="B21" s="5" t="s">
         <v>22</v>
       </c>
@@ -2723,7 +2738,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:10" s="10" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="43"/>
+      <c r="A22" s="47"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
@@ -2748,7 +2763,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:10" s="10" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="43" t="s">
+      <c r="A24" s="47" t="s">
         <v>8</v>
       </c>
       <c r="B24" s="5" t="s">
@@ -2767,7 +2782,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:10" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A25" s="43"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="5" t="s">
         <v>22</v>
       </c>
@@ -2784,54 +2799,80 @@
       <c r="G25" s="14"/>
       <c r="J25" s="32"/>
     </row>
-    <row r="26" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="43"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
+    <row r="26" spans="1:10" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
+      <c r="A26" s="47"/>
+      <c r="B26" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="E26" s="4"/>
-      <c r="F26" s="6"/>
+      <c r="F26" s="6">
+        <v>1</v>
+      </c>
       <c r="G26" s="14"/>
       <c r="J26" s="32"/>
     </row>
-    <row r="27" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="43"/>
-      <c r="B27" s="4"/>
+    <row r="27" spans="1:10" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
+      <c r="A27" s="47"/>
+      <c r="B27" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
+      <c r="D27" s="4" t="s">
+        <v>76</v>
+      </c>
       <c r="E27" s="4"/>
-      <c r="F27" s="6"/>
+      <c r="F27" s="6">
+        <v>0.5</v>
+      </c>
       <c r="G27" s="14"/>
-    </row>
-    <row r="28" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A28" s="31">
-        <v>45799</v>
-      </c>
-      <c r="B28" s="34"/>
-      <c r="C28" s="34"/>
-      <c r="D28" s="34"/>
-      <c r="E28" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="F28" s="18">
-        <f>SUM(F24:F27)</f>
-        <v>1.5</v>
+      <c r="J27" s="32"/>
+    </row>
+    <row r="28" spans="1:10" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
+      <c r="A28" s="47"/>
+      <c r="B28" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F28" s="6">
+        <v>0.5</v>
       </c>
       <c r="G28" s="14"/>
-    </row>
-    <row r="29" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A29" s="43" t="s">
-        <v>9</v>
-      </c>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
+      <c r="J28" s="32"/>
+    </row>
+    <row r="29" spans="1:10" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+      <c r="A29" s="47"/>
+      <c r="B29" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>78</v>
+      </c>
       <c r="E29" s="4"/>
-      <c r="F29" s="6"/>
+      <c r="F29" s="6">
+        <v>3.5</v>
+      </c>
       <c r="G29" s="14"/>
-    </row>
-    <row r="30" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A30" s="43"/>
+      <c r="J29" s="32"/>
+    </row>
+    <row r="30" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="47"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -2840,16 +2881,25 @@
       <c r="G30" s="14"/>
     </row>
     <row r="31" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A31" s="43"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="6"/>
+      <c r="A31" s="31">
+        <v>45799</v>
+      </c>
+      <c r="B31" s="34"/>
+      <c r="C31" s="34"/>
+      <c r="D31" s="34"/>
+      <c r="E31" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" s="18">
+        <f>SUM(F24:F30)</f>
+        <v>7</v>
+      </c>
       <c r="G31" s="14"/>
     </row>
-    <row r="32" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="43"/>
+    <row r="32" spans="1:10" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A32" s="47" t="s">
+        <v>9</v>
+      </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
@@ -2857,52 +2907,79 @@
       <c r="F32" s="6"/>
       <c r="G32" s="14"/>
     </row>
-    <row r="33" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="31">
+    <row r="33" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A33" s="47"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="14"/>
+    </row>
+    <row r="34" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A34" s="47"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="14"/>
+    </row>
+    <row r="35" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="47"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="14"/>
+    </row>
+    <row r="36" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="31">
         <v>45800</v>
       </c>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="20" t="s">
+      <c r="B36" s="19"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="F33" s="21">
-        <f>SUM(F29:F32)</f>
+      <c r="F36" s="21">
+        <f>SUM(F32:F35)</f>
         <v>0</v>
       </c>
-      <c r="G33" s="14"/>
-    </row>
-    <row r="34" spans="1:7" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="39" t="s">
+      <c r="G36" s="14"/>
+    </row>
+    <row r="37" spans="1:7" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="B34" s="39"/>
-      <c r="C34" s="39"/>
-      <c r="D34" s="39"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17" t="s">
+      <c r="B37" s="43"/>
+      <c r="C37" s="43"/>
+      <c r="D37" s="43"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="G34" s="22">
-        <f>F11+F17+F23+F28+F33</f>
-        <v>22.5</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="36" t="s">
+      <c r="G37" s="22">
+        <f>F11+F17+F23+F31+F36</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="B35" s="37"/>
-      <c r="C35" s="37"/>
-      <c r="D35" s="37"/>
-      <c r="E35" s="37"/>
-      <c r="F35" s="37"/>
-      <c r="G35" s="38"/>
+      <c r="B38" s="41"/>
+      <c r="C38" s="41"/>
+      <c r="D38" s="41"/>
+      <c r="E38" s="41"/>
+      <c r="F38" s="41"/>
+      <c r="G38" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="A38:G38"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="B3:B4"/>
@@ -2911,11 +2988,11 @@
     <mergeCell ref="A5:A10"/>
     <mergeCell ref="A12:A16"/>
     <mergeCell ref="A18:A22"/>
-    <mergeCell ref="A24:A27"/>
-    <mergeCell ref="A29:A32"/>
-    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A24:A30"/>
+    <mergeCell ref="A32:A35"/>
+    <mergeCell ref="A37:D37"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F33">
+  <conditionalFormatting sqref="F5:F36">
     <cfRule type="containsText" dxfId="23" priority="1" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",F5)))</formula>
     </cfRule>
@@ -2923,12 +3000,12 @@
       <formula>NOT(ISERROR(SEARCH("En cours",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G34">
+  <conditionalFormatting sqref="G37">
     <cfRule type="containsText" dxfId="21" priority="3" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",G34)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",G37)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="20" priority="4" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",G34)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",G37)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2973,19 +3050,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="45" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -2996,11 +3073,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="41"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -3009,7 +3086,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="46" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -3020,7 +3097,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="43"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -3029,7 +3106,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="43"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -3038,7 +3115,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="43"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -3047,7 +3124,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="43"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="E9" s="4"/>
@@ -3055,7 +3132,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="43"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -3080,7 +3157,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="47" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -3091,7 +3168,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="43"/>
+      <c r="A13" s="47"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -3100,7 +3177,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="43"/>
+      <c r="A14" s="47"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -3109,7 +3186,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="43"/>
+      <c r="A15" s="47"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -3134,7 +3211,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="47" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -3145,7 +3222,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="43"/>
+      <c r="A18" s="47"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -3154,7 +3231,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="43"/>
+      <c r="A19" s="47"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -3163,7 +3240,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="43"/>
+      <c r="A20" s="47"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -3188,7 +3265,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="47" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -3199,7 +3276,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="43"/>
+      <c r="A23" s="47"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -3208,7 +3285,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="43"/>
+      <c r="A24" s="47"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -3217,7 +3294,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="43"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -3242,7 +3319,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="47" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -3253,7 +3330,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="43"/>
+      <c r="A28" s="47"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -3262,7 +3339,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="43"/>
+      <c r="A29" s="47"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -3271,7 +3348,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="43"/>
+      <c r="A30" s="47"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -3296,12 +3373,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="39" t="s">
+      <c r="A32" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="39"/>
-      <c r="C32" s="39"/>
-      <c r="D32" s="39"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -3312,23 +3389,18 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="36" t="s">
+      <c r="A33" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="37"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="37"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="38"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A5:A10"/>
@@ -3336,6 +3408,11 @@
     <mergeCell ref="A17:A20"/>
     <mergeCell ref="A22:A25"/>
     <mergeCell ref="A27:A30"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F31">
     <cfRule type="containsText" dxfId="19" priority="1" operator="containsText" text="Terminé">
@@ -3393,19 +3470,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="45" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -3416,11 +3493,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="41"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -3429,7 +3506,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="46" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -3440,7 +3517,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="43"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -3449,7 +3526,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="43"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -3458,7 +3535,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="43"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -3467,7 +3544,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="43"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -3476,7 +3553,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="43"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -3501,7 +3578,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="47" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -3512,7 +3589,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="43"/>
+      <c r="A13" s="47"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -3521,7 +3598,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="43"/>
+      <c r="A14" s="47"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -3530,7 +3607,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="43"/>
+      <c r="A15" s="47"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -3555,7 +3632,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="47" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -3566,7 +3643,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="43"/>
+      <c r="A18" s="47"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -3575,7 +3652,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="43"/>
+      <c r="A19" s="47"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -3584,7 +3661,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="43"/>
+      <c r="A20" s="47"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -3609,7 +3686,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="47" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -3620,7 +3697,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="43"/>
+      <c r="A23" s="47"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -3629,7 +3706,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="43"/>
+      <c r="A24" s="47"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -3638,7 +3715,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="43"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -3663,7 +3740,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="47" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -3674,7 +3751,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="43"/>
+      <c r="A28" s="47"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -3683,7 +3760,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="43"/>
+      <c r="A29" s="47"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -3692,7 +3769,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="43"/>
+      <c r="A30" s="47"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -3717,12 +3794,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="39" t="s">
+      <c r="A32" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="39"/>
-      <c r="C32" s="39"/>
-      <c r="D32" s="39"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -3733,23 +3810,18 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="36" t="s">
+      <c r="A33" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="37"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="37"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="38"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A5:A10"/>
@@ -3757,6 +3829,11 @@
     <mergeCell ref="A17:A20"/>
     <mergeCell ref="A22:A25"/>
     <mergeCell ref="A27:A30"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F31">
     <cfRule type="containsText" dxfId="15" priority="1" operator="containsText" text="Terminé">
@@ -3814,19 +3891,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="45" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -3837,11 +3914,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="41"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -3850,7 +3927,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="46" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -3861,7 +3938,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="43"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -3870,7 +3947,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="43"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -3879,7 +3956,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="43"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -3888,7 +3965,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="43"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -3897,7 +3974,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="43"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -3922,7 +3999,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="47" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -3933,7 +4010,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="43"/>
+      <c r="A13" s="47"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -3942,7 +4019,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="43"/>
+      <c r="A14" s="47"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -3951,7 +4028,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="43"/>
+      <c r="A15" s="47"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -3976,7 +4053,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="47" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -3987,7 +4064,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="43"/>
+      <c r="A18" s="47"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -3996,7 +4073,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="43"/>
+      <c r="A19" s="47"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -4005,7 +4082,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="43"/>
+      <c r="A20" s="47"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -4030,7 +4107,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="47" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -4041,7 +4118,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="43"/>
+      <c r="A23" s="47"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -4050,7 +4127,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="43"/>
+      <c r="A24" s="47"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -4059,7 +4136,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="43"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -4084,7 +4161,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="47" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -4095,7 +4172,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="43"/>
+      <c r="A28" s="47"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -4104,7 +4181,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="43"/>
+      <c r="A29" s="47"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -4113,7 +4190,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="43"/>
+      <c r="A30" s="47"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -4138,12 +4215,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="39" t="s">
+      <c r="A32" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="39"/>
-      <c r="C32" s="39"/>
-      <c r="D32" s="39"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -4154,15 +4231,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="36" t="s">
+      <c r="A33" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="37"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="37"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="38"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -4237,19 +4314,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="45" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -4260,11 +4337,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="41"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -4273,7 +4350,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="46" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -4284,7 +4361,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="43"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -4293,7 +4370,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="43"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -4302,7 +4379,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="43"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -4311,7 +4388,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="43"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -4320,7 +4397,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="43"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -4345,7 +4422,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="47" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -4356,7 +4433,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="43"/>
+      <c r="A13" s="47"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -4365,7 +4442,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="43"/>
+      <c r="A14" s="47"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -4374,7 +4451,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="43"/>
+      <c r="A15" s="47"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -4399,7 +4476,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="47" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -4410,7 +4487,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="43"/>
+      <c r="A18" s="47"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -4419,7 +4496,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="43"/>
+      <c r="A19" s="47"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -4428,7 +4505,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="43"/>
+      <c r="A20" s="47"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -4453,7 +4530,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="47" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -4464,7 +4541,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="43"/>
+      <c r="A23" s="47"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -4473,7 +4550,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="43"/>
+      <c r="A24" s="47"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -4482,7 +4559,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="43"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -4507,7 +4584,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="47" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -4518,7 +4595,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="43"/>
+      <c r="A28" s="47"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -4527,7 +4604,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="43"/>
+      <c r="A29" s="47"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -4536,7 +4613,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="43"/>
+      <c r="A30" s="47"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -4561,12 +4638,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="39" t="s">
+      <c r="A32" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="39"/>
-      <c r="C32" s="39"/>
-      <c r="D32" s="39"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -4577,15 +4654,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="36" t="s">
+      <c r="A33" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="37"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="37"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="38"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -4658,19 +4735,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="45" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -4681,11 +4758,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="41"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -4694,7 +4771,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="46" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -4705,7 +4782,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="43"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -4714,7 +4791,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="43"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="E7" s="5"/>
@@ -4722,7 +4799,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="43"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -4731,7 +4808,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="43"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -4740,7 +4817,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="43"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -4765,7 +4842,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="47" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -4776,7 +4853,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="43"/>
+      <c r="A13" s="47"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -4785,7 +4862,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="43"/>
+      <c r="A14" s="47"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -4794,7 +4871,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="43"/>
+      <c r="A15" s="47"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -4819,7 +4896,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="47" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -4830,7 +4907,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="43"/>
+      <c r="A18" s="47"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -4839,7 +4916,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="43"/>
+      <c r="A19" s="47"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -4848,7 +4925,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="43"/>
+      <c r="A20" s="47"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -4873,7 +4950,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="47" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -4884,7 +4961,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="43"/>
+      <c r="A23" s="47"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -4893,7 +4970,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="43"/>
+      <c r="A24" s="47"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -4902,7 +4979,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="43"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -4927,7 +5004,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="47" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -4938,7 +5015,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="43"/>
+      <c r="A28" s="47"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -4947,7 +5024,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="43"/>
+      <c r="A29" s="47"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -4956,7 +5033,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="43"/>
+      <c r="A30" s="47"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -4981,12 +5058,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="39" t="s">
+      <c r="A32" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="39"/>
-      <c r="C32" s="39"/>
-      <c r="D32" s="39"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -4997,15 +5074,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="36" t="s">
+      <c r="A33" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="37"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="37"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="38"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
montage et ESSAIE de programmation du prototype
j'ai fait la mise en service et j'ai monter le proto puis j'ai essayer de le faire marcher
</commit_message>
<xml_diff>
--- a/jeu_du_moulin_boura/rpt/jeu-du-moulin-bourquenouda-rpt-journal.xlsx
+++ b/jeu_du_moulin_boura/rpt/jeu-du-moulin-bourquenouda-rpt-journal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bourquenouda01\OneDrive - EDUETATFR\PHIE\jeu_du_moulin_alexandre_bourquenoud\jeu_du_moulin_2025_boura\jeu_du_moulin_boura\rpt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1ECA0CE-96E2-4441-9910-690B43543D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A869703D-C38E-420F-8D0F-C459E030BBC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="s1" sheetId="8" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="104">
   <si>
     <t>Date</t>
   </si>
@@ -431,6 +431,18 @@
   </si>
   <si>
     <t>Plus il y a de LEDs allumer plus on voit le clignotement dû à la matrice et je ne peux pas contrôler le nombre maximum en jeux (18) sur le prototype, donc je ne peux pas encore mesurer les fréquences d'allumage des LEDs maximum. Je dois donc attendre mon prototype pour que je puisse faire les tests</t>
+  </si>
+  <si>
+    <t>Rédaction de la protocole de mise en service.</t>
+  </si>
+  <si>
+    <t>Montage et début de la mise en service du PCB</t>
+  </si>
+  <si>
+    <t>changements dans le programme pour convenir à l'IC utilisé sur mon proto</t>
+  </si>
+  <si>
+    <t>Cette semaine c'est aussi bien passé malgré le fait que j'ai commencé le montage plus tard que prévu à cause du jours férié…</t>
   </si>
 </sst>
 </file>
@@ -717,6 +729,18 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -752,18 +776,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1443,19 +1455,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="45" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -1466,11 +1478,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="41"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -1479,7 +1491,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" s="10" customFormat="1" ht="78.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="46" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -1500,7 +1512,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A6" s="43"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
@@ -1517,7 +1529,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="43"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="5" t="s">
         <v>22</v>
       </c>
@@ -1534,7 +1546,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="43"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="5" t="s">
         <v>22</v>
       </c>
@@ -1551,7 +1563,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A9" s="43"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="5" t="s">
         <v>22</v>
       </c>
@@ -1568,7 +1580,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" s="10" customFormat="1" ht="78.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="43"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="5" t="s">
         <v>22</v>
       </c>
@@ -1587,7 +1599,7 @@
       <c r="G10" s="14"/>
     </row>
     <row r="11" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A11" s="43"/>
+      <c r="A11" s="47"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -1612,7 +1624,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A13" s="46" t="s">
+      <c r="A13" s="50" t="s">
         <v>5</v>
       </c>
       <c r="B13" s="5" t="s">
@@ -1631,7 +1643,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A14" s="47"/>
+      <c r="A14" s="51"/>
       <c r="B14" s="5" t="s">
         <v>22</v>
       </c>
@@ -1648,7 +1660,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="47"/>
+      <c r="A15" s="51"/>
       <c r="B15" s="5" t="s">
         <v>22</v>
       </c>
@@ -1665,7 +1677,7 @@
       <c r="G15" s="14"/>
     </row>
     <row r="16" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A16" s="47"/>
+      <c r="A16" s="51"/>
       <c r="B16" s="5" t="s">
         <v>22</v>
       </c>
@@ -1682,7 +1694,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A17" s="47"/>
+      <c r="A17" s="51"/>
       <c r="B17" s="5" t="s">
         <v>22</v>
       </c>
@@ -1699,7 +1711,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="47"/>
+      <c r="A18" s="51"/>
       <c r="B18" s="5" t="s">
         <v>22</v>
       </c>
@@ -1716,7 +1728,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A19" s="47"/>
+      <c r="A19" s="51"/>
       <c r="B19" s="5"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -1741,7 +1753,7 @@
       <c r="G20" s="14"/>
     </row>
     <row r="21" spans="1:7" s="10" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
-      <c r="A21" s="42" t="s">
+      <c r="A21" s="46" t="s">
         <v>7</v>
       </c>
       <c r="B21" s="5" t="s">
@@ -1760,7 +1772,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="43"/>
+      <c r="A22" s="47"/>
       <c r="B22" s="5" t="s">
         <v>22</v>
       </c>
@@ -1777,7 +1789,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A23" s="43"/>
+      <c r="A23" s="47"/>
       <c r="B23" s="5" t="s">
         <v>22</v>
       </c>
@@ -1794,7 +1806,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A24" s="43"/>
+      <c r="A24" s="47"/>
       <c r="B24" s="5" t="s">
         <v>22</v>
       </c>
@@ -1811,7 +1823,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A25" s="43"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="5" t="s">
         <v>22</v>
       </c>
@@ -1828,7 +1840,7 @@
       <c r="G25" s="14"/>
     </row>
     <row r="26" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="43"/>
+      <c r="A26" s="47"/>
       <c r="B26" s="5" t="s">
         <v>22</v>
       </c>
@@ -1847,7 +1859,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A27" s="43"/>
+      <c r="A27" s="47"/>
       <c r="B27" s="5" t="s">
         <v>22</v>
       </c>
@@ -1880,7 +1892,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A29" s="42" t="s">
+      <c r="A29" s="46" t="s">
         <v>8</v>
       </c>
       <c r="B29" s="5" t="s">
@@ -1899,7 +1911,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A30" s="43"/>
+      <c r="A30" s="47"/>
       <c r="B30" s="5" t="s">
         <v>22</v>
       </c>
@@ -1918,7 +1930,7 @@
       <c r="G30" s="14"/>
     </row>
     <row r="31" spans="1:7" s="10" customFormat="1" ht="90" x14ac:dyDescent="0.2">
-      <c r="A31" s="43"/>
+      <c r="A31" s="47"/>
       <c r="B31" s="5" t="s">
         <v>22</v>
       </c>
@@ -1937,7 +1949,7 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" s="10" customFormat="1" ht="78.75" x14ac:dyDescent="0.2">
-      <c r="A32" s="43"/>
+      <c r="A32" s="47"/>
       <c r="B32" s="5" t="s">
         <v>22</v>
       </c>
@@ -1954,7 +1966,7 @@
       <c r="G32" s="14"/>
     </row>
     <row r="33" spans="1:7" s="10" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
-      <c r="A33" s="43"/>
+      <c r="A33" s="47"/>
       <c r="B33" s="5" t="s">
         <v>22</v>
       </c>
@@ -1971,7 +1983,7 @@
       <c r="G33" s="14"/>
     </row>
     <row r="34" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A34" s="43"/>
+      <c r="A34" s="47"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
@@ -1998,7 +2010,7 @@
       <c r="G35" s="14"/>
     </row>
     <row r="36" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A36" s="42" t="s">
+      <c r="A36" s="46" t="s">
         <v>9</v>
       </c>
       <c r="B36" s="5" t="s">
@@ -2017,7 +2029,7 @@
       <c r="G36" s="14"/>
     </row>
     <row r="37" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A37" s="43"/>
+      <c r="A37" s="47"/>
       <c r="B37" s="5" t="s">
         <v>22</v>
       </c>
@@ -2034,7 +2046,7 @@
       <c r="G37" s="14"/>
     </row>
     <row r="38" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A38" s="43"/>
+      <c r="A38" s="47"/>
       <c r="B38" s="5" t="s">
         <v>22</v>
       </c>
@@ -2053,7 +2065,7 @@
       <c r="G38" s="14"/>
     </row>
     <row r="39" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A39" s="43"/>
+      <c r="A39" s="47"/>
       <c r="B39" s="5" t="s">
         <v>22</v>
       </c>
@@ -2072,7 +2084,7 @@
       <c r="G39" s="14"/>
     </row>
     <row r="40" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A40" s="43"/>
+      <c r="A40" s="47"/>
       <c r="B40" s="5"/>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
@@ -2097,12 +2109,12 @@
       <c r="G41" s="14"/>
     </row>
     <row r="42" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="41" t="s">
+      <c r="A42" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="B42" s="44"/>
-      <c r="C42" s="44"/>
-      <c r="D42" s="45"/>
+      <c r="B42" s="48"/>
+      <c r="C42" s="48"/>
+      <c r="D42" s="49"/>
       <c r="E42" s="17"/>
       <c r="F42" s="17" t="s">
         <v>12</v>
@@ -2113,36 +2125,36 @@
       </c>
     </row>
     <row r="43" spans="1:7" s="10" customFormat="1" ht="82.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="36" t="s">
+      <c r="A43" s="40" t="s">
         <v>62</v>
       </c>
-      <c r="B43" s="37"/>
-      <c r="C43" s="37"/>
-      <c r="D43" s="37"/>
-      <c r="E43" s="37"/>
-      <c r="F43" s="37"/>
-      <c r="G43" s="38"/>
+      <c r="B43" s="41"/>
+      <c r="C43" s="41"/>
+      <c r="D43" s="41"/>
+      <c r="E43" s="41"/>
+      <c r="F43" s="41"/>
+      <c r="G43" s="42"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="48"/>
-      <c r="B46" s="48"/>
-      <c r="C46" s="49"/>
-      <c r="D46" s="48"/>
-      <c r="E46" s="48"/>
+      <c r="A46" s="37"/>
+      <c r="B46" s="37"/>
+      <c r="C46" s="39"/>
+      <c r="D46" s="37"/>
+      <c r="E46" s="37"/>
       <c r="F46" s="23"/>
       <c r="G46" s="23"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="48"/>
-      <c r="B47" s="48"/>
-      <c r="C47" s="49"/>
-      <c r="D47" s="48"/>
-      <c r="E47" s="48"/>
+      <c r="A47" s="37"/>
+      <c r="B47" s="37"/>
+      <c r="C47" s="39"/>
+      <c r="D47" s="37"/>
+      <c r="E47" s="37"/>
       <c r="F47" s="23"/>
       <c r="G47" s="23"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="50"/>
+      <c r="A48" s="36"/>
       <c r="B48" s="25"/>
       <c r="C48" s="25"/>
       <c r="D48" s="25"/>
@@ -2151,7 +2163,7 @@
       <c r="G48" s="10"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="50"/>
+      <c r="A49" s="36"/>
       <c r="B49" s="25"/>
       <c r="C49" s="25"/>
       <c r="D49" s="25"/>
@@ -2160,7 +2172,7 @@
       <c r="G49" s="10"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="50"/>
+      <c r="A50" s="36"/>
       <c r="B50" s="25"/>
       <c r="C50" s="25"/>
       <c r="D50" s="25"/>
@@ -2169,7 +2181,7 @@
       <c r="G50" s="10"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="50"/>
+      <c r="A51" s="36"/>
       <c r="B51" s="25"/>
       <c r="C51" s="25"/>
       <c r="D51" s="25"/>
@@ -2178,7 +2190,7 @@
       <c r="G51" s="10"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="50"/>
+      <c r="A52" s="36"/>
       <c r="B52" s="25"/>
       <c r="C52" s="25"/>
       <c r="D52" s="25"/>
@@ -2187,7 +2199,7 @@
       <c r="G52" s="10"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="50"/>
+      <c r="A53" s="36"/>
       <c r="B53" s="25"/>
       <c r="C53" s="25"/>
       <c r="D53" s="25"/>
@@ -2205,7 +2217,7 @@
       <c r="G54" s="10"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="50"/>
+      <c r="A55" s="36"/>
       <c r="B55" s="25"/>
       <c r="C55" s="25"/>
       <c r="D55" s="25"/>
@@ -2214,7 +2226,7 @@
       <c r="G55" s="10"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="50"/>
+      <c r="A56" s="36"/>
       <c r="B56" s="25"/>
       <c r="C56" s="25"/>
       <c r="D56" s="25"/>
@@ -2223,7 +2235,7 @@
       <c r="G56" s="10"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="50"/>
+      <c r="A57" s="36"/>
       <c r="B57" s="25"/>
       <c r="C57" s="25"/>
       <c r="D57" s="25"/>
@@ -2232,7 +2244,7 @@
       <c r="G57" s="10"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="50"/>
+      <c r="A58" s="36"/>
       <c r="B58" s="25"/>
       <c r="C58" s="25"/>
       <c r="D58" s="25"/>
@@ -2250,7 +2262,7 @@
       <c r="G59" s="10"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="50"/>
+      <c r="A60" s="36"/>
       <c r="B60" s="25"/>
       <c r="C60" s="25"/>
       <c r="D60" s="25"/>
@@ -2259,7 +2271,7 @@
       <c r="G60" s="10"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="50"/>
+      <c r="A61" s="36"/>
       <c r="B61" s="25"/>
       <c r="C61" s="25"/>
       <c r="D61" s="25"/>
@@ -2268,7 +2280,7 @@
       <c r="G61" s="10"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="50"/>
+      <c r="A62" s="36"/>
       <c r="B62" s="25"/>
       <c r="C62" s="25"/>
       <c r="D62" s="25"/>
@@ -2277,7 +2289,7 @@
       <c r="G62" s="10"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="50"/>
+      <c r="A63" s="36"/>
       <c r="B63" s="25"/>
       <c r="C63" s="25"/>
       <c r="D63" s="25"/>
@@ -2295,7 +2307,7 @@
       <c r="G64" s="10"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" s="50"/>
+      <c r="A65" s="36"/>
       <c r="B65" s="25"/>
       <c r="C65" s="25"/>
       <c r="D65" s="25"/>
@@ -2304,7 +2316,7 @@
       <c r="G65" s="10"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" s="50"/>
+      <c r="A66" s="36"/>
       <c r="B66" s="25"/>
       <c r="C66" s="25"/>
       <c r="D66" s="25"/>
@@ -2313,7 +2325,7 @@
       <c r="G66" s="10"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" s="50"/>
+      <c r="A67" s="36"/>
       <c r="B67" s="25"/>
       <c r="C67" s="25"/>
       <c r="D67" s="25"/>
@@ -2322,7 +2334,7 @@
       <c r="G67" s="10"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" s="50"/>
+      <c r="A68" s="36"/>
       <c r="B68" s="25"/>
       <c r="C68" s="25"/>
       <c r="D68" s="25"/>
@@ -2340,7 +2352,7 @@
       <c r="G69" s="10"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" s="50"/>
+      <c r="A70" s="36"/>
       <c r="B70" s="25"/>
       <c r="C70" s="25"/>
       <c r="D70" s="25"/>
@@ -2349,7 +2361,7 @@
       <c r="G70" s="10"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" s="50"/>
+      <c r="A71" s="36"/>
       <c r="B71" s="25"/>
       <c r="C71" s="25"/>
       <c r="D71" s="25"/>
@@ -2358,7 +2370,7 @@
       <c r="G71" s="10"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" s="50"/>
+      <c r="A72" s="36"/>
       <c r="B72" s="25"/>
       <c r="C72" s="25"/>
       <c r="D72" s="25"/>
@@ -2367,7 +2379,7 @@
       <c r="G72" s="10"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A73" s="50"/>
+      <c r="A73" s="36"/>
       <c r="B73" s="25"/>
       <c r="C73" s="25"/>
       <c r="D73" s="25"/>
@@ -2385,37 +2397,25 @@
       <c r="G74" s="10"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" s="48"/>
-      <c r="B75" s="48"/>
-      <c r="C75" s="48"/>
-      <c r="D75" s="48"/>
+      <c r="A75" s="37"/>
+      <c r="B75" s="37"/>
+      <c r="C75" s="37"/>
+      <c r="D75" s="37"/>
       <c r="E75" s="27"/>
       <c r="F75" s="27"/>
       <c r="G75" s="28"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" s="51"/>
-      <c r="B76" s="51"/>
-      <c r="C76" s="51"/>
-      <c r="D76" s="51"/>
-      <c r="E76" s="51"/>
-      <c r="F76" s="51"/>
-      <c r="G76" s="51"/>
+      <c r="A76" s="38"/>
+      <c r="B76" s="38"/>
+      <c r="C76" s="38"/>
+      <c r="D76" s="38"/>
+      <c r="E76" s="38"/>
+      <c r="F76" s="38"/>
+      <c r="G76" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A48:A53"/>
-    <mergeCell ref="A75:D75"/>
-    <mergeCell ref="A76:G76"/>
-    <mergeCell ref="A55:A58"/>
-    <mergeCell ref="A60:A63"/>
-    <mergeCell ref="A65:A68"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A46:A47"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="E46:E47"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
@@ -2428,6 +2428,18 @@
     <mergeCell ref="A36:A40"/>
     <mergeCell ref="A42:D42"/>
     <mergeCell ref="A13:A19"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="E46:E47"/>
+    <mergeCell ref="A48:A53"/>
+    <mergeCell ref="A75:D75"/>
+    <mergeCell ref="A76:G76"/>
+    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="A60:A63"/>
+    <mergeCell ref="A65:A68"/>
+    <mergeCell ref="A70:A73"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F16 F20:F41">
     <cfRule type="containsText" dxfId="31" priority="1" operator="containsText" text="Terminé">
@@ -2508,19 +2520,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="45" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -2531,11 +2543,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="41"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -2544,7 +2556,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="46" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -2563,7 +2575,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A6" s="43"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
@@ -2580,7 +2592,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" s="10" customFormat="1" ht="90" x14ac:dyDescent="0.2">
-      <c r="A7" s="43"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="5" t="s">
         <v>22</v>
       </c>
@@ -2599,7 +2611,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="43"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="5" t="s">
         <v>22</v>
       </c>
@@ -2616,7 +2628,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" s="10" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="43"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -2625,7 +2637,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="43"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -2650,7 +2662,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="47" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="5" t="s">
@@ -2669,7 +2681,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" s="10" customFormat="1" ht="67.5" x14ac:dyDescent="0.2">
-      <c r="A13" s="43"/>
+      <c r="A13" s="47"/>
       <c r="B13" s="5" t="s">
         <v>22</v>
       </c>
@@ -2686,7 +2698,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A14" s="43"/>
+      <c r="A14" s="47"/>
       <c r="B14" s="5" t="s">
         <v>22</v>
       </c>
@@ -2703,7 +2715,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A15" s="43"/>
+      <c r="A15" s="47"/>
       <c r="B15" s="5" t="s">
         <v>22</v>
       </c>
@@ -2720,7 +2732,7 @@
       <c r="G15" s="14"/>
     </row>
     <row r="16" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="43"/>
+      <c r="A16" s="47"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
@@ -2745,7 +2757,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:10" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A18" s="43" t="s">
+      <c r="A18" s="47" t="s">
         <v>7</v>
       </c>
       <c r="B18" s="5" t="s">
@@ -2765,7 +2777,7 @@
       <c r="J18" s="32"/>
     </row>
     <row r="19" spans="1:10" s="10" customFormat="1" ht="146.25" x14ac:dyDescent="0.2">
-      <c r="A19" s="43"/>
+      <c r="A19" s="47"/>
       <c r="B19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2782,7 +2794,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:10" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A20" s="43"/>
+      <c r="A20" s="47"/>
       <c r="B20" s="5" t="s">
         <v>22</v>
       </c>
@@ -2799,7 +2811,7 @@
       <c r="G20" s="14"/>
     </row>
     <row r="21" spans="1:10" s="10" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="43"/>
+      <c r="A21" s="47"/>
       <c r="B21" s="5" t="s">
         <v>22</v>
       </c>
@@ -2816,7 +2828,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:10" s="10" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="43"/>
+      <c r="A22" s="47"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
@@ -2841,7 +2853,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:10" s="10" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="43" t="s">
+      <c r="A24" s="47" t="s">
         <v>8</v>
       </c>
       <c r="B24" s="5" t="s">
@@ -2860,7 +2872,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:10" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A25" s="43"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="5" t="s">
         <v>22</v>
       </c>
@@ -2878,7 +2890,7 @@
       <c r="J25" s="32"/>
     </row>
     <row r="26" spans="1:10" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="43"/>
+      <c r="A26" s="47"/>
       <c r="B26" s="5" t="s">
         <v>22</v>
       </c>
@@ -2896,7 +2908,7 @@
       <c r="J26" s="32"/>
     </row>
     <row r="27" spans="1:10" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A27" s="43"/>
+      <c r="A27" s="47"/>
       <c r="B27" s="5" t="s">
         <v>22</v>
       </c>
@@ -2912,7 +2924,7 @@
       <c r="J27" s="32"/>
     </row>
     <row r="28" spans="1:10" s="10" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
-      <c r="A28" s="43"/>
+      <c r="A28" s="47"/>
       <c r="B28" s="5" t="s">
         <v>22</v>
       </c>
@@ -2932,7 +2944,7 @@
       <c r="J28" s="32"/>
     </row>
     <row r="29" spans="1:10" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A29" s="43"/>
+      <c r="A29" s="47"/>
       <c r="B29" s="5" t="s">
         <v>22</v>
       </c>
@@ -2950,7 +2962,7 @@
       <c r="J29" s="32"/>
     </row>
     <row r="30" spans="1:10" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="43"/>
+      <c r="A30" s="47"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -2975,7 +2987,7 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:10" s="10" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
-      <c r="A32" s="43" t="s">
+      <c r="A32" s="47" t="s">
         <v>9</v>
       </c>
       <c r="B32" s="5" t="s">
@@ -2994,7 +3006,7 @@
       <c r="G32" s="14"/>
     </row>
     <row r="33" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A33" s="43"/>
+      <c r="A33" s="47"/>
       <c r="B33" s="5" t="s">
         <v>22</v>
       </c>
@@ -3009,7 +3021,7 @@
       <c r="G33" s="14"/>
     </row>
     <row r="34" spans="1:7" s="10" customFormat="1" ht="101.25" x14ac:dyDescent="0.2">
-      <c r="A34" s="43"/>
+      <c r="A34" s="47"/>
       <c r="B34" s="5" t="s">
         <v>22</v>
       </c>
@@ -3028,7 +3040,7 @@
       <c r="G34" s="14"/>
     </row>
     <row r="35" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A35" s="43"/>
+      <c r="A35" s="47"/>
       <c r="B35" s="5" t="s">
         <v>22</v>
       </c>
@@ -3047,7 +3059,7 @@
       <c r="G35" s="14"/>
     </row>
     <row r="36" spans="1:7" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A36" s="43"/>
+      <c r="A36" s="47"/>
       <c r="B36" s="5" t="s">
         <v>22</v>
       </c>
@@ -3064,7 +3076,7 @@
       <c r="G36" s="14"/>
     </row>
     <row r="37" spans="1:7" s="10" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
-      <c r="A37" s="43"/>
+      <c r="A37" s="47"/>
       <c r="B37" s="5" t="s">
         <v>22</v>
       </c>
@@ -3081,7 +3093,7 @@
       <c r="G37" s="14"/>
     </row>
     <row r="38" spans="1:7" s="10" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="43"/>
+      <c r="A38" s="47"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
@@ -3106,12 +3118,12 @@
       <c r="G39" s="14"/>
     </row>
     <row r="40" spans="1:7" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="39" t="s">
+      <c r="A40" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="B40" s="39"/>
-      <c r="C40" s="39"/>
-      <c r="D40" s="39"/>
+      <c r="B40" s="43"/>
+      <c r="C40" s="43"/>
+      <c r="D40" s="43"/>
       <c r="E40" s="17"/>
       <c r="F40" s="17" t="s">
         <v>12</v>
@@ -3122,15 +3134,15 @@
       </c>
     </row>
     <row r="41" spans="1:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="36" t="s">
+      <c r="A41" s="40" t="s">
         <v>87</v>
       </c>
-      <c r="B41" s="37"/>
-      <c r="C41" s="37"/>
-      <c r="D41" s="37"/>
-      <c r="E41" s="37"/>
-      <c r="F41" s="37"/>
-      <c r="G41" s="38"/>
+      <c r="B41" s="41"/>
+      <c r="C41" s="41"/>
+      <c r="D41" s="41"/>
+      <c r="E41" s="41"/>
+      <c r="F41" s="41"/>
+      <c r="G41" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -3170,13 +3182,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B49AD842-BAFE-408E-B382-9CD2E9A5A143}">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="30.85546875" customWidth="1"/>
     <col min="3" max="3" width="9.5703125" customWidth="1"/>
     <col min="4" max="4" width="50.85546875" customWidth="1"/>
-    <col min="5" max="5" width="76.28515625" customWidth="1"/>
+    <col min="5" max="5" width="30" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -3206,19 +3218,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="45" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -3229,11 +3241,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="41"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -3242,7 +3254,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="46" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -3261,7 +3273,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A6" s="43"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
@@ -3280,7 +3292,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="43"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
@@ -3293,7 +3305,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="43"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -3302,7 +3314,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="43"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="E9" s="4"/>
@@ -3310,7 +3322,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="43"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -3335,7 +3347,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="47" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="5" t="s">
@@ -3354,7 +3366,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="43"/>
+      <c r="A13" s="47"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="5" t="s">
@@ -3369,7 +3381,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" ht="67.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="43"/>
+      <c r="A14" s="47"/>
       <c r="B14" s="5" t="s">
         <v>22</v>
       </c>
@@ -3388,7 +3400,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="43"/>
+      <c r="A15" s="47"/>
       <c r="B15" s="5" t="s">
         <v>22</v>
       </c>
@@ -3405,7 +3417,7 @@
       <c r="G15" s="14"/>
     </row>
     <row r="16" spans="1:7" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="43"/>
+      <c r="A16" s="47"/>
       <c r="B16" s="5" t="s">
         <v>22</v>
       </c>
@@ -3422,7 +3434,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="43"/>
+      <c r="A17" s="47"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
@@ -3447,7 +3459,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="43" t="s">
+      <c r="A19" s="47" t="s">
         <v>7</v>
       </c>
       <c r="B19" s="5" t="s">
@@ -3466,7 +3478,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="43"/>
+      <c r="A20" s="47"/>
       <c r="B20" s="5" t="s">
         <v>22</v>
       </c>
@@ -3483,7 +3495,7 @@
       <c r="G20" s="14"/>
     </row>
     <row r="21" spans="1:7" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A21" s="43"/>
+      <c r="A21" s="47"/>
       <c r="B21" s="5" t="s">
         <v>22</v>
       </c>
@@ -3502,7 +3514,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="43"/>
+      <c r="A22" s="47"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
@@ -3527,7 +3539,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="43" t="s">
+      <c r="A24" s="47" t="s">
         <v>8</v>
       </c>
       <c r="B24" s="4" t="s">
@@ -3540,7 +3552,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="43"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -3549,7 +3561,7 @@
       <c r="G25" s="14"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="43"/>
+      <c r="A26" s="47"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
@@ -3558,7 +3570,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="43"/>
+      <c r="A27" s="47"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
       <c r="D27" s="4"/>
@@ -3576,109 +3588,164 @@
       <c r="E28" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="F28" s="18">
-        <f>SUM(F24:F27)</f>
-        <v>0</v>
-      </c>
+      <c r="F28" s="18"/>
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="43" t="s">
+      <c r="A29" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
+      <c r="B29" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="E29" s="4"/>
-      <c r="F29" s="6"/>
+      <c r="F29" s="13">
+        <v>0.2</v>
+      </c>
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="43"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
+      <c r="A30" s="47"/>
+      <c r="B30" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>100</v>
+      </c>
       <c r="E30" s="4"/>
-      <c r="F30" s="6"/>
+      <c r="F30" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G30" s="14"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="43"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
+      <c r="A31" s="47"/>
+      <c r="B31" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>94</v>
+      </c>
       <c r="E31" s="4"/>
-      <c r="F31" s="6"/>
+      <c r="F31" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G31" s="14"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="43"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
+    <row r="32" spans="1:7" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A32" s="47"/>
+      <c r="B32" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>102</v>
+      </c>
       <c r="E32" s="4"/>
-      <c r="F32" s="6"/>
+      <c r="F32" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G32" s="14"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="31">
+      <c r="A33" s="47"/>
+      <c r="B33" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E33" s="4"/>
+      <c r="F33" s="6">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="G33" s="14"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="47"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="14"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="31">
         <v>45807</v>
       </c>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="20" t="s">
+      <c r="B35" s="19"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="19"/>
+      <c r="E35" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="F33" s="21">
-        <f>SUM(F29:F32)</f>
-        <v>0</v>
-      </c>
-      <c r="G33" s="14"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="39" t="s">
+      <c r="F35" s="21">
+        <f>SUM(F29:F34)</f>
+        <v>7</v>
+      </c>
+      <c r="G35" s="14"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="B34" s="39"/>
-      <c r="C34" s="39"/>
-      <c r="D34" s="39"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17" t="s">
+      <c r="B36" s="43"/>
+      <c r="C36" s="43"/>
+      <c r="D36" s="43"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="G34" s="22">
-        <f>F11+F18+F23+F28+F33</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="36" t="s">
-        <v>15</v>
-      </c>
-      <c r="B35" s="37"/>
-      <c r="C35" s="37"/>
-      <c r="D35" s="37"/>
-      <c r="E35" s="37"/>
-      <c r="F35" s="37"/>
-      <c r="G35" s="38"/>
+      <c r="G36" s="22">
+        <f>F11+F18+F23+F28+F35</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="B37" s="41"/>
+      <c r="C37" s="41"/>
+      <c r="D37" s="41"/>
+      <c r="E37" s="41"/>
+      <c r="F37" s="41"/>
+      <c r="G37" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A5:A10"/>
+    <mergeCell ref="A12:A17"/>
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="A24:A27"/>
+    <mergeCell ref="A29:A34"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="E3:E4"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="A35:G35"/>
-    <mergeCell ref="A5:A10"/>
-    <mergeCell ref="A12:A17"/>
-    <mergeCell ref="A19:A22"/>
-    <mergeCell ref="A24:A27"/>
-    <mergeCell ref="A29:A32"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F33">
+  <conditionalFormatting sqref="F5:F35">
     <cfRule type="containsText" dxfId="19" priority="1" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",F5)))</formula>
     </cfRule>
@@ -3686,15 +3753,16 @@
       <formula>NOT(ISERROR(SEARCH("En cours",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G34">
+  <conditionalFormatting sqref="G36">
     <cfRule type="containsText" dxfId="17" priority="5" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",G34)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",G36)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="16" priority="6" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",G34)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",G36)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3734,19 +3802,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="45" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -3757,11 +3825,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="41"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -3770,7 +3838,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="46" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -3781,7 +3849,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="43"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -3790,7 +3858,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="43"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -3799,7 +3867,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="43"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -3808,7 +3876,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="43"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -3817,7 +3885,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="43"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -3842,7 +3910,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="47" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -3853,7 +3921,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="43"/>
+      <c r="A13" s="47"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -3862,7 +3930,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="43"/>
+      <c r="A14" s="47"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -3871,7 +3939,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="43"/>
+      <c r="A15" s="47"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -3896,7 +3964,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="47" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -3907,7 +3975,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="43"/>
+      <c r="A18" s="47"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -3916,7 +3984,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="43"/>
+      <c r="A19" s="47"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -3925,7 +3993,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="43"/>
+      <c r="A20" s="47"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -3950,7 +4018,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="47" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -3961,7 +4029,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="43"/>
+      <c r="A23" s="47"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -3970,7 +4038,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="43"/>
+      <c r="A24" s="47"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -3979,7 +4047,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="43"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -4004,7 +4072,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="47" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -4015,7 +4083,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="43"/>
+      <c r="A28" s="47"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -4024,7 +4092,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="43"/>
+      <c r="A29" s="47"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -4033,7 +4101,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="43"/>
+      <c r="A30" s="47"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -4058,12 +4126,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="39" t="s">
+      <c r="A32" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="39"/>
-      <c r="C32" s="39"/>
-      <c r="D32" s="39"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -4074,23 +4142,18 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="36" t="s">
+      <c r="A33" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="37"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="37"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="38"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A5:A10"/>
@@ -4098,6 +4161,11 @@
     <mergeCell ref="A17:A20"/>
     <mergeCell ref="A22:A25"/>
     <mergeCell ref="A27:A30"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F31">
     <cfRule type="containsText" dxfId="15" priority="1" operator="containsText" text="Terminé">
@@ -4155,19 +4223,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="45" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -4178,11 +4246,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="41"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -4191,7 +4259,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="46" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -4202,7 +4270,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="43"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -4211,7 +4279,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="43"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -4220,7 +4288,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="43"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -4229,7 +4297,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="43"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -4238,7 +4306,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="43"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -4263,7 +4331,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="47" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -4274,7 +4342,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="43"/>
+      <c r="A13" s="47"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -4283,7 +4351,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="43"/>
+      <c r="A14" s="47"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -4292,7 +4360,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="43"/>
+      <c r="A15" s="47"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -4317,7 +4385,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="47" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -4328,7 +4396,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="43"/>
+      <c r="A18" s="47"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -4337,7 +4405,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="43"/>
+      <c r="A19" s="47"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -4346,7 +4414,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="43"/>
+      <c r="A20" s="47"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -4371,7 +4439,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="47" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -4382,7 +4450,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="43"/>
+      <c r="A23" s="47"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -4391,7 +4459,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="43"/>
+      <c r="A24" s="47"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -4400,7 +4468,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="43"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -4425,7 +4493,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="47" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -4436,7 +4504,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="43"/>
+      <c r="A28" s="47"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -4445,7 +4513,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="43"/>
+      <c r="A29" s="47"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -4454,7 +4522,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="43"/>
+      <c r="A30" s="47"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -4479,12 +4547,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="39" t="s">
+      <c r="A32" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="39"/>
-      <c r="C32" s="39"/>
-      <c r="D32" s="39"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -4495,15 +4563,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="36" t="s">
+      <c r="A33" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="37"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="37"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="38"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -4578,19 +4646,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="45" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -4601,11 +4669,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="41"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -4614,7 +4682,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="46" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -4625,7 +4693,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="43"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -4634,7 +4702,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="43"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -4643,7 +4711,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="43"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -4652,7 +4720,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="43"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -4661,7 +4729,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="43"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -4686,7 +4754,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="47" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -4697,7 +4765,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="43"/>
+      <c r="A13" s="47"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -4706,7 +4774,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="43"/>
+      <c r="A14" s="47"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -4715,7 +4783,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="43"/>
+      <c r="A15" s="47"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -4740,7 +4808,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="47" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -4751,7 +4819,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="43"/>
+      <c r="A18" s="47"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -4760,7 +4828,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="43"/>
+      <c r="A19" s="47"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -4769,7 +4837,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="43"/>
+      <c r="A20" s="47"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -4794,7 +4862,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="47" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -4805,7 +4873,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="43"/>
+      <c r="A23" s="47"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -4814,7 +4882,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="43"/>
+      <c r="A24" s="47"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -4823,7 +4891,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="43"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -4848,7 +4916,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="47" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -4859,7 +4927,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="43"/>
+      <c r="A28" s="47"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -4868,7 +4936,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="43"/>
+      <c r="A29" s="47"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -4877,7 +4945,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="43"/>
+      <c r="A30" s="47"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -4902,12 +4970,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="39" t="s">
+      <c r="A32" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="39"/>
-      <c r="C32" s="39"/>
-      <c r="D32" s="39"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -4918,15 +4986,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="36" t="s">
+      <c r="A33" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="37"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="37"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="38"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -4999,19 +5067,19 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="45" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -5022,11 +5090,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="41"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -5035,7 +5103,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="46" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5"/>
@@ -5046,7 +5114,7 @@
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="43"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -5055,7 +5123,7 @@
       <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="43"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="E7" s="5"/>
@@ -5063,7 +5131,7 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="43"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -5072,7 +5140,7 @@
       <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="43"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -5081,7 +5149,7 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="43"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -5106,7 +5174,7 @@
       <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="47" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="4"/>
@@ -5117,7 +5185,7 @@
       <c r="G12" s="14"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="43"/>
+      <c r="A13" s="47"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -5126,7 +5194,7 @@
       <c r="G13" s="14"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="43"/>
+      <c r="A14" s="47"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -5135,7 +5203,7 @@
       <c r="G14" s="14"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="43"/>
+      <c r="A15" s="47"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -5160,7 +5228,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="47" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="4"/>
@@ -5171,7 +5239,7 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="43"/>
+      <c r="A18" s="47"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -5180,7 +5248,7 @@
       <c r="G18" s="14"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="43"/>
+      <c r="A19" s="47"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -5189,7 +5257,7 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="43"/>
+      <c r="A20" s="47"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -5214,7 +5282,7 @@
       <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="47" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="4"/>
@@ -5225,7 +5293,7 @@
       <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="43"/>
+      <c r="A23" s="47"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -5234,7 +5302,7 @@
       <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="43"/>
+      <c r="A24" s="47"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -5243,7 +5311,7 @@
       <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="43"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -5268,7 +5336,7 @@
       <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="47" t="s">
         <v>9</v>
       </c>
       <c r="B27" s="4"/>
@@ -5279,7 +5347,7 @@
       <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="43"/>
+      <c r="A28" s="47"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -5288,7 +5356,7 @@
       <c r="G28" s="14"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="43"/>
+      <c r="A29" s="47"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -5297,7 +5365,7 @@
       <c r="G29" s="14"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="43"/>
+      <c r="A30" s="47"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -5322,12 +5390,12 @@
       <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="39" t="s">
+      <c r="A32" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="39"/>
-      <c r="C32" s="39"/>
-      <c r="D32" s="39"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43"/>
       <c r="E32" s="17"/>
       <c r="F32" s="17" t="s">
         <v>12</v>
@@ -5338,15 +5406,15 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="36" t="s">
+      <c r="A33" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="37"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="37"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="38"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>